<commit_message>
Localize question bank v2 authoring draft
</commit_message>
<xml_diff>
--- a/docs/question_bank_v2/question_bank_v2_authoring_draft.xlsx
+++ b/docs/question_bank_v2/question_bank_v2_authoring_draft.xlsx
@@ -642,7 +642,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Fast opener about why a House should listen to host instructions and role signals before acting.</t>
+          <t>Быстрый стартовый вопрос: почему Дому важно слушать ведущего и сигналы ролей перед действием.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="AA2" s="3" t="inlineStr">
         <is>
-          <t>Convert into concise true/false.</t>
+          <t>Сделать коротким вопросом true/false.</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Simple question about when gold matters during requests, House choices, and table strategy.</t>
+          <t>Простой вопрос о том, когда золото влияет на заявки, решения Дома и игровую стратегию.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="AA3" s="3" t="inlineStr">
         <is>
-          <t>Reinforce gold without changing economy rules.</t>
+          <t>Закрепляет экономику без изменения правил.</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Players identify a familiar table or bar object from a close-up image.</t>
+          <t>Игроки узнают знакомый предмет со стола или бара по крупному фрагменту изображения.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="AA4" s="3" t="inlineStr">
         <is>
-          <t>First low-stakes image; must be readable from far tables.</t>
+          <t>Первый лёгкий визуальный вопрос; картинка должна читаться с дальних столов.</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Question asks which House role is best suited to negotiate with another House.</t>
+          <t>Вопрос о том, какая роль Дома лучше всего подходит для переговоров с другим Домом.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="AA5" s="3" t="inlineStr">
         <is>
-          <t>Keep playful; avoid feeling like a rules test.</t>
+          <t>Оставить живым и игровым, не превращать в экзамен по правилам.</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Light food misconception question with a surprising but safe explanation.</t>
+          <t>Лёгкий вопрос о распространённом мифе про еду с неожиданным, но безопасным объяснением.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="AA6" s="3" t="inlineStr">
         <is>
-          <t>Needs concrete fact later.</t>
+          <t>Нужен конкретный проверенный факт.</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Question about what to do when phone, TV, and host timing feel out of sync.</t>
+          <t>Вопрос о том, что делать, если телефон, ТВ и ведущий будто показывают разные стадии.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="AA7" s="3" t="inlineStr">
         <is>
-          <t>Consider moving to host script instead of scored question.</t>
+          <t>Лучше перенести в речь ведущего, если звучит слишком служебно.</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Players identify what old tool or object was used for.</t>
+          <t>Игроки определяют, для чего использовался старый инструмент или предмет.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="AA8" s="3" t="inlineStr">
         <is>
-          <t>Strong visual recognition slot; source/rights check needed.</t>
+          <t>Сильный визуальный слот; нужен источник и проверка прав.</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1477,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Question about meaning of a common menu, bar, or service symbol.</t>
+          <t>Вопрос о значении распространённого символа в меню, баре или сервисе.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="AA9" s="3" t="inlineStr">
         <is>
-          <t>Can use venue-inspired but not false brand claim.</t>
+          <t>Можно вдохновляться площадкой, но не делать неподтверждённое утверждение о бренде.</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Players infer product category from a cropped old-style advertisement or poster fragment.</t>
+          <t>Игроки по фрагменту старой рекламы или плаката угадывают категорию продукта.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="AA10" s="3" t="inlineStr">
         <is>
-          <t>Rights/source risk; do not finalize without approval.</t>
+          <t>Риск по правам на источник; не финализировать без проверки.</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Object whose name or purpose is often mistaken; players choose real use.</t>
+          <t>Предмет с часто ошибочным названием или назначением: игроки выбирают реальное применение.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="AA11" s="3" t="inlineStr">
         <is>
-          <t>Could become image if asset appears.</t>
+          <t>Можно позже превратить в визуальный вопрос, если найдётся хороший ассет.</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1836,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Local map/sign/orientation clue question, pending exact Kurgan/Sobranie reference.</t>
+          <t>Локальный вопрос по карте, вывеске или ориентиру; точная курганская/собранийская привязка ещё не утверждена.</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="AA12" s="3" t="inlineStr">
         <is>
-          <t>Needs Victor/local approval before wording.</t>
+          <t>Нужно одобрение Виктора и проверка локального факта.</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Social-reading question: what table behavior signals a House is ready to negotiate.</t>
+          <t>Вопрос на социальное чтение: какое поведение за столом показывает, что Дом готов к переговорам.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="AA13" s="3" t="inlineStr">
         <is>
-          <t>Supports Diplomacy without adding mechanics.</t>
+          <t>Поддерживает дипломатию без добавления новых механик.</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Question about how glass/serving shape can change perception of a drink.</t>
+          <t>Вопрос о том, как форма бокала или подачи может менять восприятие напитка.</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="AA14" s="3" t="inlineStr">
         <is>
-          <t>Keep non-alcohol or 18+ safe.</t>
+          <t>Держать в безалкогольной или безопасной для 18+ зоне.</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Delayed image clue where players infer answer from a broad visual detail.</t>
+          <t>Отложенная визуальная подсказка: игроки делают вывод по крупной детали изображения.</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="AA15" s="3" t="inlineStr">
         <is>
-          <t>Avoid tiny details; TV readability required.</t>
+          <t>Не использовать мелкие детали; нужна проверка читаемости на ТВ.</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Players choose the most plausible origin story of a common object or ritual.</t>
+          <t>Игроки выбирают наиболее правдоподобную историю происхождения привычного предмета или ритуала.</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="AA16" s="3" t="inlineStr">
         <is>
-          <t>Needs strong options and fact check.</t>
+          <t>Нужны сильные варианты ответа и фактчек.</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Food texture or ingredient close-up; players infer dish/category.</t>
+          <t>Крупный фрагмент еды или ингредиента: игроки угадывают блюдо или категорию.</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="AA17" s="3" t="inlineStr">
         <is>
-          <t>Good bar-energy visual; avoid gross ambiguity.</t>
+          <t>Хороший барный визуал; избегать неприятной или слишком неоднозначной картинки.</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Host plays short manual audio; players identify mood, era, or context.</t>
+          <t>Ведущий вручную включает короткий аудиофрагмент; игроки определяют настроение, эпоху или контекст.</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -2604,7 +2604,7 @@
       <c r="P18" s="3" t="inlineStr"/>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>Host/operator plays manually outside the app; fallback text is needed.</t>
+          <t>Ведущий/оператор запускает вручную вне приложения; нужен текстовый fallback.</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
@@ -2654,7 +2654,7 @@
       </c>
       <c r="AA18" s="3" t="inlineStr">
         <is>
-          <t>Manual/offline only; source/legal/fallback required.</t>
+          <t>Только вручную/офлайн; нужны источник, правовая проверка и fallback.</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Strategy/social question about which negotiation move most likely signals a bluff.</t>
+          <t>Стратегический вопрос: какой переговорный ход больше всего похож на блеф.</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="AA19" s="3" t="inlineStr">
         <is>
-          <t>Keep playful, not accusatory.</t>
+          <t>Держать игровым и лёгким, без личных обвинений.</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Text-first question; reveal image explains unexpected object or fact after answer.</t>
+          <t>Сначала текстовый вопрос, затем картинка на раскрытии объясняет неожиданный предмет или факт.</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="AA20" s="3" t="inlineStr">
         <is>
-          <t>Strong staged reveal candidate.</t>
+          <t>Сильный кандидат для staged reveal.</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Local/Kurgan-flavored fact question pending exact approved reference.</t>
+          <t>Локальный вопрос с курганским оттенком; точная ссылка будет добавлена после утверждения.</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="AA21" s="3" t="inlineStr">
         <is>
-          <t>Needs local truth check before wording.</t>
+          <t>Нужна проверка локальной правды.</t>
         </is>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Pattern/arrangement image; players identify what changed or what it is used for.</t>
+          <t>Изображение с паттерном или расположением: игроки определяют, что изменилось или для чего это используется.</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="AA22" s="3" t="inlineStr">
         <is>
-          <t>Must be visible from far tables.</t>
+          <t>Должно быть видно с дальних столов.</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Host plays/describes a short sound; players identify instrument family or setting.</t>
+          <t>Ведущий вручную включает или описывает короткий звук; игроки определяют семейство инструмента или ситуацию.</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -3213,7 +3213,7 @@
       <c r="P23" s="3" t="inlineStr"/>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>Host/operator plays manually outside the app; fallback text is needed.</t>
+          <t>Ведущий/оператор запускает вручную вне приложения; нужен текстовый fallback.</t>
         </is>
       </c>
       <c r="R23" s="3" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="AA23" s="3" t="inlineStr">
         <is>
-          <t>Manual/offline only; text fallback required.</t>
+          <t>Только вручную/офлайн; нужен текстовый fallback.</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Short Court-safe factual question that can settle public tension cleanly.</t>
+          <t>Короткий судебный факт-вопрос, который можно спокойно разобрать публично.</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="AA24" s="3" t="inlineStr">
         <is>
-          <t>Keep low ambiguity.</t>
+          <t>Должен быть однозначным и легко объяснимым.</t>
         </is>
       </c>
     </row>
@@ -3413,7 +3413,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Image presented as Court evidence; players infer what it most likely proves.</t>
+          <t>Изображение как улика для Суда: игроки определяют, что оно вероятнее всего доказывает.</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="AA25" s="3" t="inlineStr">
         <is>
-          <t>Use only if simple and TV-smoked.</t>
+          <t>Использовать только если картинка простая и проверена на ТВ.</t>
         </is>
       </c>
     </row>
@@ -3538,7 +3538,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Court strategy question about safe House decision when gold is limited.</t>
+          <t>Судебный стратегический вопрос: какое решение Дома безопаснее при ограниченном золоте.</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -3622,7 +3622,7 @@
       </c>
       <c r="AA26" s="3" t="inlineStr">
         <is>
-          <t>Must not imply automatic gold/resource mutation.</t>
+          <t>Не должно подразумевать автоматическое изменение золота или ресурсов.</t>
         </is>
       </c>
     </row>
@@ -3655,7 +3655,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Short non-controversial food/bar fact suitable for Court.</t>
+          <t>Короткий нейтральный факт про еду или барную культуру для Суда.</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -3739,7 +3739,7 @@
       </c>
       <c r="AA27" s="3" t="inlineStr">
         <is>
-          <t>Avoid alcohol/legal ambiguity.</t>
+          <t>Избегать спорной алкогольной или юридической зоны.</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Court question where reveal image explains why the answer was true.</t>
+          <t>Судебный вопрос, где изображение на раскрытии объясняет, почему ответ верный.</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="AA28" s="3" t="inlineStr">
         <is>
-          <t>Reveal image, not clue-critical.</t>
+          <t>Картинка объясняет ответ, но не должна быть критичной подсказкой.</t>
         </is>
       </c>
     </row>
@@ -3897,7 +3897,7 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Role/Court prompt about who should speak for a House in a public dispute.</t>
+          <t>Ролевой судебный промпт: кто должен говорить от имени Дома в публичном споре.</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="AA29" s="3" t="inlineStr">
         <is>
-          <t>Consider manual host prompt instead of import.</t>
+          <t>Возможно, лучше оставить ручным промптом ведущего, а не импортировать.</t>
         </is>
       </c>
     </row>
@@ -4014,7 +4014,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Clear final-round general culture question with low ambiguity.</t>
+          <t>Понятный финальный вопрос общей культуры с низкой неоднозначностью.</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -4098,7 +4098,7 @@
       </c>
       <c r="AA30" s="3" t="inlineStr">
         <is>
-          <t>Needs strong explanation.</t>
+          <t>Нужно сильное объяснение для раскрытия.</t>
         </is>
       </c>
     </row>
@@ -4131,7 +4131,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Fully tested final image clue for decisive tension.</t>
+          <t>Финальная визуальная подсказка для напряжённого решающего вопроса.</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="AA31" s="3" t="inlineStr">
         <is>
-          <t>Use only if excellent and smoke-passed.</t>
+          <t>Использовать только если картинка отличная и прошла smoke.</t>
         </is>
       </c>
     </row>
@@ -4256,7 +4256,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Optional final manual audio/mood clue with text fallback.</t>
+          <t>Опциональная финальная ручная аудиоподсказка с текстовым fallback.</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -4298,7 +4298,7 @@
       <c r="P32" s="3" t="inlineStr"/>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>Host/operator plays manually outside the app; fallback text is needed.</t>
+          <t>Ведущий/оператор запускает вручную вне приложения; нужен текстовый fallback.</t>
         </is>
       </c>
       <c r="R32" s="3" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="AA32" s="3" t="inlineStr">
         <is>
-          <t>Optional; no runtime audio.</t>
+          <t>Опционально; runtime audio не используется.</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Strategic final prompt about risk vs safe points for a House.</t>
+          <t>Финальный стратегический промпт о выборе риска или безопасных очков для Дома.</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="AA33" s="3" t="inlineStr">
         <is>
-          <t>Decide if scored question or host discussion.</t>
+          <t>Решить, это scored question или обсуждение ведущего.</t>
         </is>
       </c>
     </row>
@@ -4498,7 +4498,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Very short duel-ready question about identifying familiar object or fact.</t>
+          <t>Очень короткий дуэльный вопрос про знакомый предмет или факт.</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="AA34" s="3" t="inlineStr">
         <is>
-          <t>Keep extremely short.</t>
+          <t>Сделать максимально коротким.</t>
         </is>
       </c>
     </row>
@@ -4615,7 +4615,7 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Fast true/false Duel question with immediate understandable answer.</t>
+          <t>Быстрый true/false вопрос для Дуэли с мгновенно понятным ответом.</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -4699,7 +4699,7 @@
       </c>
       <c r="AA35" s="3" t="inlineStr">
         <is>
-          <t>No ambiguity.</t>
+          <t>Без неоднозначности.</t>
         </is>
       </c>
     </row>
@@ -4732,7 +4732,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Optional image-based Duel question if the image is instantly readable.</t>
+          <t>Опциональный визуальный вопрос для Дуэли, если картинка считывается мгновенно.</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="AA36" s="3" t="inlineStr">
         <is>
-          <t>Likely cut unless very clear.</t>
+          <t>Скорее всего вырезать, если картинка не очевидна.</t>
         </is>
       </c>
     </row>
@@ -4857,7 +4857,7 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Host manual pacing moment for tie, pause, or table reset.</t>
+          <t>Ручной момент ведущего для ничьей, паузы или перезапуска стола.</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="AA37" s="3" t="inlineStr">
         <is>
-          <t>Probably not imported.</t>
+          <t>Вероятно, не импортировать.</t>
         </is>
       </c>
     </row>
@@ -4974,7 +4974,7 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Plain reserve food/drink culture question with no media dependency.</t>
+          <t>Резервный простой вопрос про еду или напитки без медиа-зависимости.</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="AA38" s="3" t="inlineStr">
         <is>
-          <t>Backup if media fails.</t>
+          <t>Запасной вопрос на случай проблем с медиа.</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Strange everyday-history reserve question.</t>
+          <t>Резервный вопрос про странную историю повседневной вещи.</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="AA39" s="3" t="inlineStr">
         <is>
-          <t>Needs fact check before use.</t>
+          <t>Нужен фактчек перед использованием.</t>
         </is>
       </c>
     </row>
@@ -5208,7 +5208,7 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Backup image clue if another visual question is rejected.</t>
+          <t>Резервная визуальная подсказка, если другой визуальный вопрос будет отклонён.</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="AA40" s="3" t="inlineStr">
         <is>
-          <t>Optional reserve asset.</t>
+          <t>Опциональный резервный ассет.</t>
         </is>
       </c>
     </row>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Reserve question about negotiation/social behavior with no personal accusation.</t>
+          <t>Резервный вопрос про переговоры или социальное поведение без личных обвинений.</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
@@ -5417,7 +5417,7 @@
       </c>
       <c r="AA41" s="3" t="inlineStr">
         <is>
-          <t>Supports Diplomacy vibe.</t>
+          <t>Поддерживает атмосферу дипломатии.</t>
         </is>
       </c>
     </row>
@@ -5450,7 +5450,7 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Court-safe reserve question for tie or disputed moment.</t>
+          <t>Резервный безопасный вопрос для Суда, ничьей или спорного момента.</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="AA42" s="3" t="inlineStr">
         <is>
-          <t>Robust fallback.</t>
+          <t>Надёжный fallback.</t>
         </is>
       </c>
     </row>
@@ -5567,7 +5567,7 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Backup manual audio moment with text-only fallback.</t>
+          <t>Резервный ручной аудиомомент с текстовым fallback.</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
@@ -5609,7 +5609,7 @@
       <c r="P43" s="3" t="inlineStr"/>
       <c r="Q43" s="3" t="inlineStr">
         <is>
-          <t>Host/operator plays manually outside the app; fallback text is needed.</t>
+          <t>Ведущий/оператор запускает вручную вне приложения; нужен текстовый fallback.</t>
         </is>
       </c>
       <c r="R43" s="3" t="inlineStr">
@@ -5659,7 +5659,7 @@
       </c>
       <c r="AA43" s="3" t="inlineStr">
         <is>
-          <t>Use only if source/device/fallback are ready.</t>
+          <t>Использовать только если готовы источник, устройство и fallback.</t>
         </is>
       </c>
     </row>
@@ -5692,7 +5692,7 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>Reserve local/Kurgan/Sobranie placeholder pending approval.</t>
+          <t>Резервная локальная курганская/собранийская идея до утверждения.</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="AA44" s="3" t="inlineStr">
         <is>
-          <t>Do not finalize without local check.</t>
+          <t>Не финализировать без локальной проверки.</t>
         </is>
       </c>
     </row>
@@ -5809,7 +5809,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>Reserve object trivia without image dependency.</t>
+          <t>Резервный вопрос про предмет без зависимости от картинки.</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="AA45" s="3" t="inlineStr">
         <is>
-          <t>Can become image later if needed.</t>
+          <t>Можно позже сделать визуальным, если понадобится.</t>
         </is>
       </c>
     </row>
@@ -5926,7 +5926,7 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>Clean final/tie reserve question with no media and no ambiguity.</t>
+          <t>Чистый резервный финальный или тай-брейк вопрос без медиа и неоднозначности.</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
@@ -6010,7 +6010,7 @@
       </c>
       <c r="AA46" s="3" t="inlineStr">
         <is>
-          <t>For final backup.</t>
+          <t>Для финального запаса.</t>
         </is>
       </c>
     </row>
@@ -6043,7 +6043,7 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Reserve role-understanding question for player clarity.</t>
+          <t>Резервный вопрос на понимание ролей, если за столами будет путаница.</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="AA47" s="3" t="inlineStr">
         <is>
-          <t>Useful if table confusion appears.</t>
+          <t>Полезен при слабом понимании ролей.</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Backup reveal image explaining a surprising answer after reveal.</t>
+          <t>Резервная картинка-раскрытие, объясняющая неожиданный ответ после reveal.</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
@@ -6252,7 +6252,7 @@
       </c>
       <c r="AA48" s="3" t="inlineStr">
         <is>
-          <t>Use only if asset is easy and ready.</t>
+          <t>Использовать только если ассет легко подготовить.</t>
         </is>
       </c>
     </row>
@@ -6285,7 +6285,7 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Host-choice emergency pacing, tie, or failed-media replacement moment.</t>
+          <t>Ручной аварийный момент ведущего для темпа, ничьей или замены провалившегося медиа.</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
@@ -6369,7 +6369,7 @@
       </c>
       <c r="AA49" s="3" t="inlineStr">
         <is>
-          <t>Manual only; likely not imported.</t>
+          <t>Только вручную; скорее всего не импортировать.</t>
         </is>
       </c>
     </row>
@@ -6486,7 +6486,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>object close-up / table detail</t>
+          <t>крупный план предмета на столе/барной детали</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -6511,7 +6511,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Easy first visual; must be obvious from far tables.</t>
+          <t>Лёгкий первый визуал; должен быть очевиден с дальних столов.</t>
         </is>
       </c>
     </row>
@@ -6543,7 +6543,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>historical/old object</t>
+          <t>исторический или старый предмет</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -6568,7 +6568,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Strong recognition slot; use public-safe source.</t>
+          <t>Сильный слот на узнавание; нужен безопасный публичный источник.</t>
         </is>
       </c>
     </row>
@@ -6600,7 +6600,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>old ad/poster fragment</t>
+          <t>фрагмент старой рекламы или плаката</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -6625,7 +6625,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Rights-sensitive; use only if source is safe.</t>
+          <t>Чувствительно к правам; использовать только при безопасном источнике.</t>
         </is>
       </c>
     </row>
@@ -6657,7 +6657,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>map/detail/local sign</t>
+          <t>карта, локальная вывеска или деталь ориентира</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Local/Kurgan/Sobranie placeholder; requires Victor approval.</t>
+          <t>Локальный placeholder; требуется утверждение Виктора.</t>
         </is>
       </c>
     </row>
@@ -6714,7 +6714,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>what changed / hidden detail</t>
+          <t>картинка “что изменилось?” или скрытая деталь</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -6739,7 +6739,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Must not depend on tiny visual details.</t>
+          <t>Не должна зависеть от мелких деталей.</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>food/drink close-up</t>
+          <t>крупный план еды или напитка</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -6796,7 +6796,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Good bar-energy image; avoid gross ambiguity.</t>
+          <t>Барный визуал; избегать неприятной неоднозначности.</t>
         </is>
       </c>
     </row>
@@ -6828,7 +6828,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>reveal object/explanation</t>
+          <t>картинка-объяснение для раскрытия</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Image should explain answer after reveal.</t>
+          <t>Изображение объясняет ответ после reveal.</t>
         </is>
       </c>
     </row>
@@ -6885,7 +6885,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>visual pattern / arrangement</t>
+          <t>визуальный паттерн или расположение</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -6910,7 +6910,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Must be readable from far tables.</t>
+          <t>Должно читаться с дальних столов.</t>
         </is>
       </c>
     </row>
@@ -6942,7 +6942,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>visual evidence for Court</t>
+          <t>визуальная улика для Суда</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Court image must be simple and non-controversial.</t>
+          <t>Судебное изображение должно быть простым и не провоцировать спор.</t>
         </is>
       </c>
     </row>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>symbol/logo-style reveal</t>
+          <t>символ или псевдо-логотип для раскрытия</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -7024,7 +7024,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Logo/symbol trap; no real brand misuse.</t>
+          <t>Символическая ловушка; не использовать реальные бренды без прав.</t>
         </is>
       </c>
     </row>
@@ -7056,7 +7056,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>final visual clue</t>
+          <t>финальная визуальная подсказка</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -7081,7 +7081,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Use only if polished and TV-smoke-passed.</t>
+          <t>Использовать только если картинка отполирована и проверена на ТВ.</t>
         </is>
       </c>
     </row>
@@ -7113,7 +7113,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>duel-safe fast visual</t>
+          <t>быстрый дуэльный визуал</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -7138,7 +7138,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Optional; likely cut unless instantly readable.</t>
+          <t>Опционально; скорее всего вырезать, если не считывается мгновенно.</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>reserve image clue</t>
+          <t>резервная визуальная подсказка</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -7195,7 +7195,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Reserve visual if another asset is rejected.</t>
+          <t>Резервный визуал, если другой ассет отклонён.</t>
         </is>
       </c>
     </row>
@@ -7290,7 +7290,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Host plays short instrumental/mood fragment outside app.</t>
+          <t>Ведущий вручную включает короткий инструментальный или атмосферный фрагмент вне приложения.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Use text-only mood/context question.</t>
+          <t>Использовать текстовый вопрос про настроение или контекст.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -7315,7 +7315,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Primary manual audio moment.</t>
+          <t>Основной ручной аудиомомент.</t>
         </is>
       </c>
     </row>
@@ -7337,7 +7337,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Host plays/describes a short sound or instrument moment manually.</t>
+          <t>Ведущий вручную включает или описывает короткий звук/инструментальный момент.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Read text description and ask instrument-family question.</t>
+          <t>Зачитать текстовое описание и спросить про семейство инструмента.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -7362,7 +7362,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Use only if source/fallback is simple.</t>
+          <t>Использовать только если источник и fallback простые.</t>
         </is>
       </c>
     </row>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Host plays final atmosphere/audio clue manually.</t>
+          <t>Ведущий вручную включает финальную атмосферную аудиоподсказку.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Use final text question only.</t>
+          <t>Использовать только финальный текстовый вопрос.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -7409,7 +7409,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Optional final moment; no runtime dependency.</t>
+          <t>Опциональный финальный момент; без runtime-зависимости.</t>
         </is>
       </c>
     </row>
@@ -7431,7 +7431,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Host uses backup manual audio if time/need exists.</t>
+          <t>Ведущий использует резервное аудио вручную, если есть время или необходимость.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -7446,7 +7446,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Skip and use plain reserve question.</t>
+          <t>Пропустить и взять обычный резервный вопрос.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -7456,7 +7456,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Reserve fallback only.</t>
+          <t>Только резервный fallback.</t>
         </is>
       </c>
     </row>
@@ -7573,7 +7573,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -7637,7 +7637,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Needs Victor/operator approval.</t>
+          <t>Нужно утверждение Виктора/оператора.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -7661,7 +7661,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -7705,7 +7705,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -7749,7 +7749,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -7793,7 +7793,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Needs Victor/operator approval.</t>
+          <t>Нужно утверждение Виктора/оператора.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
@@ -7817,7 +7817,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
@@ -7841,7 +7841,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Needs fact check.</t>
+          <t>Нужна проверка факта.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
@@ -7889,7 +7889,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Needs manual audio source/legal/fallback decision.</t>
+          <t>Нужно решение по ручному аудио: источник, права и fallback.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
@@ -7933,7 +7933,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
@@ -7957,7 +7957,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Needs Victor/operator approval.</t>
+          <t>Нужно утверждение Виктора/оператора.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
@@ -7981,7 +7981,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
@@ -8005,7 +8005,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Needs manual audio source/legal/fallback decision.</t>
+          <t>Нужно решение по ручному аудио: источник, права и fallback.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Needs fact check.</t>
+          <t>Нужна проверка факта.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
@@ -8053,7 +8053,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
@@ -8077,7 +8077,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Needs Victor/operator approval.</t>
+          <t>Нужно утверждение Виктора/оператора.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
@@ -8101,7 +8101,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Needs fact check.</t>
+          <t>Нужна проверка факта.</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
@@ -8125,7 +8125,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
@@ -8149,7 +8149,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Needs Victor/operator approval.</t>
+          <t>Нужно утверждение Виктора/оператора.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
@@ -8173,7 +8173,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Needs fact check.</t>
+          <t>Нужна проверка факта.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
@@ -8197,7 +8197,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
@@ -8221,7 +8221,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Needs manual audio source/legal/fallback decision.</t>
+          <t>Нужно решение по ручному аудио: источник, права и fallback.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr"/>
@@ -8245,7 +8245,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Needs Victor/operator approval.</t>
+          <t>Нужно утверждение Виктора/оператора.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>
@@ -8309,7 +8309,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
@@ -8333,7 +8333,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Needs Victor/operator approval.</t>
+          <t>Нужно утверждение Виктора/оператора.</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -8355,7 +8355,11 @@
           <t>reserve</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr"/>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Резервная строка: использовать только после отбора.</t>
+        </is>
+      </c>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="inlineStr"/>
     </row>
@@ -8377,7 +8381,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Needs fact check.</t>
+          <t>Нужна проверка факта.</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
@@ -8401,7 +8405,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr"/>
@@ -8423,7 +8427,11 @@
           <t>reserve</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Резервная строка: использовать только после отбора.</t>
+        </is>
+      </c>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="3" t="inlineStr"/>
     </row>
@@ -8443,7 +8451,11 @@
           <t>reserve</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr"/>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Резервная строка: использовать только после отбора.</t>
+        </is>
+      </c>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="3" t="inlineStr"/>
     </row>
@@ -8465,7 +8477,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Needs manual audio source/legal/fallback decision.</t>
+          <t>Нужно решение по ручному аудио: источник, права и fallback.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -8489,7 +8501,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Needs Victor/operator approval.</t>
+          <t>Нужно утверждение Виктора/оператора.</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr"/>
@@ -8511,7 +8523,11 @@
           <t>reserve</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Резервная строка: использовать только после отбора.</t>
+        </is>
+      </c>
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr"/>
     </row>
@@ -8531,7 +8547,11 @@
           <t>reserve</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Резервная строка: использовать только после отбора.</t>
+        </is>
+      </c>
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="3" t="inlineStr"/>
     </row>
@@ -8551,7 +8571,11 @@
           <t>reserve</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Резервная строка: использовать только после отбора.</t>
+        </is>
+      </c>
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="3" t="inlineStr"/>
     </row>
@@ -8573,7 +8597,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Needs image asset/source/readability check.</t>
+          <t>Нужны изображение, источник, права и проверка читаемости.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr"/>
@@ -8595,7 +8619,11 @@
           <t>reserve</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Резервная строка: использовать только после отбора.</t>
+        </is>
+      </c>
       <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Fill obvious question bank v2 answers
</commit_message>
<xml_diff>
--- a/docs/question_bank_v2/question_bank_v2_authoring_draft.xlsx
+++ b/docs/question_bank_v2/question_bank_v2_authoring_draft.xlsx
@@ -1088,10 +1088,14 @@
       </c>
       <c r="H3" s="7" t="n"/>
       <c r="I3" s="7" t="n"/>
-      <c r="J3" s="9" t="n"/>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K3" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
@@ -1138,7 +1142,7 @@
       </c>
       <c r="U3" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 7. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 7. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V3" s="9" t="inlineStr">
@@ -1189,10 +1193,14 @@
       </c>
       <c r="H4" s="7" t="n"/>
       <c r="I4" s="7" t="n"/>
-      <c r="J4" s="9" t="n"/>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K4" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L4" s="9" t="inlineStr">
@@ -1234,7 +1242,7 @@
       </c>
       <c r="U4" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 8. Аудит action=keep. answer_type=true_false.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 8. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V4" s="9" t="inlineStr">
@@ -1285,10 +1293,14 @@
       </c>
       <c r="H5" s="7" t="n"/>
       <c r="I5" s="7" t="n"/>
-      <c r="J5" s="9" t="n"/>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>ложь</t>
+        </is>
+      </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L5" s="9" t="inlineStr">
@@ -1330,7 +1342,7 @@
       </c>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 9. Аудит action=keep. answer_type=true_false.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 9. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V5" s="9" t="inlineStr">
@@ -1381,10 +1393,14 @@
       </c>
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
-      <c r="J6" s="9" t="n"/>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>ложь</t>
+        </is>
+      </c>
       <c r="K6" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L6" s="9" t="inlineStr">
@@ -1426,7 +1442,7 @@
       </c>
       <c r="U6" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 10. Аудит action=keep. answer_type=true_false.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 10. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V6" s="9" t="inlineStr">
@@ -1770,10 +1786,14 @@
       </c>
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="n"/>
-      <c r="J10" s="9" t="n"/>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K10" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L10" s="9" t="inlineStr">
@@ -1815,7 +1835,7 @@
       </c>
       <c r="U10" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 14. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про астероиды каждые 2 недели.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 14. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про астероиды каждые 2 недели. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V10" s="9" t="inlineStr">
@@ -1866,10 +1886,14 @@
       </c>
       <c r="H11" s="7" t="n"/>
       <c r="I11" s="7" t="n"/>
-      <c r="J11" s="9" t="n"/>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K11" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L11" s="9" t="inlineStr">
@@ -1911,7 +1935,7 @@
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 16. Аудит action=keep. answer_type=true_false.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 16. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V11" s="9" t="inlineStr">
@@ -1962,10 +1986,14 @@
       </c>
       <c r="H12" s="7" t="n"/>
       <c r="I12" s="7" t="n"/>
-      <c r="J12" s="9" t="n"/>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K12" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L12" s="9" t="inlineStr">
@@ -2003,7 +2031,7 @@
       </c>
       <c r="U12" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 18. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить; внутренний факт подтверждён Виктором, в пицце Собрание есть халапеньо.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 18. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить; внутренний факт подтверждён Виктором, в пицце Собрание есть халапеньо. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V12" s="9" t="inlineStr">
@@ -2054,10 +2082,14 @@
       </c>
       <c r="H13" s="7" t="n"/>
       <c r="I13" s="7" t="n"/>
-      <c r="J13" s="9" t="n"/>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K13" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L13" s="9" t="inlineStr">
@@ -2099,7 +2131,7 @@
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 19. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 19. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V13" s="9" t="inlineStr">
@@ -2150,10 +2182,14 @@
       </c>
       <c r="H14" s="7" t="n"/>
       <c r="I14" s="7" t="n"/>
-      <c r="J14" s="9" t="n"/>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>ложь</t>
+        </is>
+      </c>
       <c r="K14" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L14" s="9" t="inlineStr">
@@ -2195,7 +2231,7 @@
       </c>
       <c r="U14" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 20. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 20. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V14" s="9" t="inlineStr">
@@ -2246,10 +2282,14 @@
       </c>
       <c r="H15" s="7" t="n"/>
       <c r="I15" s="7" t="n"/>
-      <c r="J15" s="9" t="n"/>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K15" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L15" s="22" t="inlineStr">
@@ -2300,7 +2340,7 @@
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 21. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Бананы.jfif; не скопирован в app/static. Решение Виктора: вопрос про бананы оставить как есть; картинку Бананы.jfif нужно кропнуть или заменить из-за чёрных полей.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 21. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Бананы.jfif; не скопирован в app/static. Решение Виктора: вопрос про бананы оставить как есть; картинку Бананы.jfif нужно кропнуть или заменить из-за чёрных полей. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V15" s="9" t="inlineStr">
@@ -2351,10 +2391,14 @@
       </c>
       <c r="H16" s="7" t="n"/>
       <c r="I16" s="7" t="n"/>
-      <c r="J16" s="9" t="n"/>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K16" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L16" s="9" t="inlineStr">
@@ -2396,7 +2440,7 @@
       </c>
       <c r="U16" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 23. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про черепах и клоакальное дыхание.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 23. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про черепах и клоакальное дыхание. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V16" s="9" t="inlineStr">
@@ -2447,10 +2491,14 @@
       </c>
       <c r="H17" s="7" t="n"/>
       <c r="I17" s="7" t="n"/>
-      <c r="J17" s="9" t="n"/>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L17" s="9" t="inlineStr">
@@ -2492,7 +2540,7 @@
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 24. Аудит action=keep. answer_type=true_false.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 24. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V17" s="9" t="inlineStr">
@@ -2543,10 +2591,14 @@
       </c>
       <c r="H18" s="7" t="n"/>
       <c r="I18" s="7" t="n"/>
-      <c r="J18" s="9" t="n"/>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>ложь</t>
+        </is>
+      </c>
       <c r="K18" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L18" s="9" t="inlineStr">
@@ -2588,7 +2640,7 @@
       </c>
       <c r="U18" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 25. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про пирамиду Хеопса и записки.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 25. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про пирамиду Хеопса и записки. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V18" s="9" t="inlineStr">
@@ -3500,10 +3552,14 @@
           <t>играет на дудочке</t>
         </is>
       </c>
-      <c r="J27" s="9" t="n"/>
+      <c r="J27" s="9" t="inlineStr">
+        <is>
+          <t>будит жителей</t>
+        </is>
+      </c>
       <c r="K27" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L27" s="10" t="inlineStr">
@@ -3554,7 +3610,7 @@
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 15. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/15. женщина будит жителей.jpeg; не скопирован в app/static. Решение Виктора: женщина будит жителей — использовать как визуальный вопрос.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 15. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/15. женщина будит жителей.jpeg; не скопирован в app/static. Решение Виктора: женщина будит жителей — использовать как визуальный вопрос. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V27" s="9" t="inlineStr">
@@ -3613,10 +3669,14 @@
           <t>продажа купальников</t>
         </is>
       </c>
-      <c r="J28" s="9" t="n"/>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>конкурс красоты</t>
+        </is>
+      </c>
       <c r="K28" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L28" s="22" t="inlineStr">
@@ -3667,7 +3727,7 @@
       </c>
       <c r="U28" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 16. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/16. конкурс красоты.png; не скопирован в app/static. Решение Виктора: конкурс красоты/лодыжки оставить только после замены картинки на чистый источник; текущая выглядит обработанной.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 16. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/16. конкурс красоты.png; не скопирован в app/static. Решение Виктора: конкурс красоты/лодыжки оставить только после замены картинки на чистый источник; текущая выглядит обработанной. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V28" s="9" t="inlineStr">
@@ -3726,10 +3786,14 @@
           <t>поднимают груз</t>
         </is>
       </c>
-      <c r="J29" s="9" t="n"/>
+      <c r="J29" s="9" t="inlineStr">
+        <is>
+          <t>спят</t>
+        </is>
+      </c>
       <c r="K29" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L29" s="10" t="inlineStr">
@@ -3780,7 +3844,7 @@
       </c>
       <c r="U29" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 17. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/17. Двухпенсовый подвес.jpg; не скопирован в app/static. Решение Виктора: двухпенсовый подвес / люди спят на верёвках — использовать как визуальный вопрос.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 17. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/17. Двухпенсовый подвес.jpg; не скопирован в app/static. Решение Виктора: двухпенсовый подвес / люди спят на верёвках — использовать как визуальный вопрос. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V29" s="9" t="inlineStr">
@@ -3839,10 +3903,14 @@
           <t>выбирали невесту</t>
         </is>
       </c>
-      <c r="J30" s="9" t="n"/>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>лечили спину</t>
+        </is>
+      </c>
       <c r="K30" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L30" s="21" t="inlineStr">
@@ -3893,7 +3961,7 @@
       </c>
       <c r="U30" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 18. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/18. Медведь).png; не скопирован в app/static. Решение Виктора: медведь лечит спину — оставить, но нужен source check.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 18. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/18. Медведь).png; не скопирован в app/static. Решение Виктора: медведь лечит спину — оставить, но нужен source check. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V30" s="9" t="inlineStr">
@@ -3952,10 +4020,14 @@
           <t>пудреница</t>
         </is>
       </c>
-      <c r="J31" s="9" t="n"/>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>уксусница</t>
+        </is>
+      </c>
       <c r="K31" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L31" s="10" t="inlineStr">
@@ -4006,7 +4078,7 @@
       </c>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 19. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/19. Уксусница.jpg; не скопирован в app/static. Решение Виктора: уксусница / коробочка с резким запахом — использовать как визуальный/object question.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 19. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/19. Уксусница.jpg; не скопирован в app/static. Решение Виктора: уксусница / коробочка с резким запахом — использовать как визуальный/object question. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V31" s="9" t="inlineStr">
@@ -4065,10 +4137,14 @@
           <t>массажер</t>
         </is>
       </c>
-      <c r="J32" s="9" t="n"/>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>фен</t>
+        </is>
+      </c>
       <c r="K32" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L32" s="9" t="inlineStr">
@@ -4110,7 +4186,7 @@
       </c>
       <c r="U32" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 20. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: предшественник фена с кипятком пока не финализировать; нужен источник/картинка.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 20. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: предшественник фена с кипятком пока не финализировать; нужен источник/картинка. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V32" s="9" t="inlineStr">
@@ -4169,10 +4245,14 @@
           <t>извлекать занозу.</t>
         </is>
       </c>
-      <c r="J33" s="9" t="n"/>
+      <c r="J33" s="9" t="inlineStr">
+        <is>
+          <t>застегивать пуговицы</t>
+        </is>
+      </c>
       <c r="K33" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L33" s="10" t="inlineStr">
@@ -4222,7 +4302,7 @@
       </c>
       <c r="U33" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 21. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: застёгиватель пуговиц / buttonhook — использовать как визуальный/object question.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 21. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: застёгиватель пуговиц / buttonhook — использовать как визуальный/object question. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V33" s="9" t="inlineStr">
@@ -4770,10 +4850,14 @@
       <c r="G39" s="7" t="n"/>
       <c r="H39" s="7" t="n"/>
       <c r="I39" s="7" t="n"/>
-      <c r="J39" s="9" t="n"/>
+      <c r="J39" s="9" t="inlineStr">
+        <is>
+          <t>микроволновая печь</t>
+        </is>
+      </c>
       <c r="K39" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L39" s="10" t="inlineStr">
@@ -4825,7 +4909,7 @@
       </c>
       <c r="U39" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 5. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Микроволновка.jpg; не скопирован в app/static. Решение Виктора: микроволновка / растаявшая конфета — использовать как визуальный вопрос.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 5. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Микроволновка.jpg; не скопирован в app/static. Решение Виктора: микроволновка / растаявшая конфета — использовать как визуальный вопрос. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V39" s="9" t="inlineStr">
@@ -5072,10 +5156,14 @@
       <c r="G42" s="7" t="n"/>
       <c r="H42" s="7" t="n"/>
       <c r="I42" s="7" t="n"/>
-      <c r="J42" s="9" t="n"/>
+      <c r="J42" s="9" t="inlineStr">
+        <is>
+          <t>точное время</t>
+        </is>
+      </c>
       <c r="K42" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L42" s="10" t="inlineStr">
@@ -5127,7 +5215,7 @@
       </c>
       <c r="U42" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 8. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Продавщица времени.jpg; не скопирован в app/static. Решение Виктора: выбрать лучший вариант между Время.jpg и Продавщица времени.jpg после просмотра.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 8. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Продавщица времени.jpg; не скопирован в app/static. Решение Виктора: выбрать лучший вариант между Время.jpg и Продавщица времени.jpg после просмотра. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V42" s="9" t="inlineStr">
@@ -6279,7 +6367,11 @@
       </c>
       <c r="K3" s="7" t="inlineStr"/>
       <c r="L3" s="7" t="inlineStr"/>
-      <c r="M3" s="7" t="inlineStr"/>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="N3" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -6340,7 +6432,7 @@
       </c>
       <c r="AA3" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 7. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 7. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6485,11 @@
       </c>
       <c r="K4" s="7" t="inlineStr"/>
       <c r="L4" s="7" t="inlineStr"/>
-      <c r="M4" s="7" t="inlineStr"/>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="N4" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -6449,7 +6545,7 @@
       </c>
       <c r="AA4" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 8. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 8. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -6502,7 +6598,11 @@
       </c>
       <c r="K5" s="7" t="inlineStr"/>
       <c r="L5" s="7" t="inlineStr"/>
-      <c r="M5" s="7" t="inlineStr"/>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>ложь</t>
+        </is>
+      </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -6558,7 +6658,7 @@
       </c>
       <c r="AA5" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 9. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 9. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -6611,7 +6711,11 @@
       </c>
       <c r="K6" s="7" t="inlineStr"/>
       <c r="L6" s="7" t="inlineStr"/>
-      <c r="M6" s="7" t="inlineStr"/>
+      <c r="M6" s="7" t="inlineStr">
+        <is>
+          <t>ложь</t>
+        </is>
+      </c>
       <c r="N6" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -6667,7 +6771,7 @@
       </c>
       <c r="AA6" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 10. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 10. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -7048,7 +7152,11 @@
       </c>
       <c r="K10" s="7" t="inlineStr"/>
       <c r="L10" s="7" t="inlineStr"/>
-      <c r="M10" s="7" t="inlineStr"/>
+      <c r="M10" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -7104,7 +7212,7 @@
       </c>
       <c r="AA10" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 14. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про астероиды каждые 2 недели. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 14. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про астероиды каждые 2 недели. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -7262,7 +7370,11 @@
       </c>
       <c r="K12" s="7" t="inlineStr"/>
       <c r="L12" s="7" t="inlineStr"/>
-      <c r="M12" s="7" t="inlineStr"/>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -7318,7 +7430,7 @@
       </c>
       <c r="AA12" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 16. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 16. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -7484,7 +7596,11 @@
       </c>
       <c r="K14" s="7" t="inlineStr"/>
       <c r="L14" s="7" t="inlineStr"/>
-      <c r="M14" s="7" t="inlineStr"/>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="N14" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -7536,7 +7652,7 @@
       </c>
       <c r="AA14" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 18. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить; внутренний факт подтверждён Виктором, в пицце Собрание есть халапеньо. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 18. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить; внутренний факт подтверждён Виктором, в пицце Собрание есть халапеньо. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -7589,7 +7705,11 @@
       </c>
       <c r="K15" s="7" t="inlineStr"/>
       <c r="L15" s="7" t="inlineStr"/>
-      <c r="M15" s="7" t="inlineStr"/>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -7645,7 +7765,7 @@
       </c>
       <c r="AA15" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 19. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 19. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -7698,7 +7818,11 @@
       </c>
       <c r="K16" s="7" t="inlineStr"/>
       <c r="L16" s="7" t="inlineStr"/>
-      <c r="M16" s="7" t="inlineStr"/>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>ложь</t>
+        </is>
+      </c>
       <c r="N16" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -7754,7 +7878,7 @@
       </c>
       <c r="AA16" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 20. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 20. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -7807,7 +7931,11 @@
       </c>
       <c r="K17" s="7" t="inlineStr"/>
       <c r="L17" s="7" t="inlineStr"/>
-      <c r="M17" s="7" t="inlineStr"/>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -7868,7 +7996,7 @@
       </c>
       <c r="AA17" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 21. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Бананы.jfif; не скопирован в app/static. Решение Виктора: вопрос про бананы оставить как есть; картинку Бананы.jfif нужно кропнуть или заменить из-за чёрных полей. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 21. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Бананы.jfif; не скопирован в app/static. Решение Виктора: вопрос про бананы оставить как есть; картинку Бананы.jfif нужно кропнуть или заменить из-за чёрных полей. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -8030,7 +8158,11 @@
       </c>
       <c r="K19" s="7" t="inlineStr"/>
       <c r="L19" s="7" t="inlineStr"/>
-      <c r="M19" s="7" t="inlineStr"/>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -8086,7 +8218,7 @@
       </c>
       <c r="AA19" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 23. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про черепах и клоакальное дыхание. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 23. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про черепах и клоакальное дыхание. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -8139,7 +8271,11 @@
       </c>
       <c r="K20" s="7" t="inlineStr"/>
       <c r="L20" s="7" t="inlineStr"/>
-      <c r="M20" s="7" t="inlineStr"/>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -8195,7 +8331,7 @@
       </c>
       <c r="AA20" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 24. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 24. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -8248,7 +8384,11 @@
       </c>
       <c r="K21" s="7" t="inlineStr"/>
       <c r="L21" s="7" t="inlineStr"/>
-      <c r="M21" s="7" t="inlineStr"/>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>ложь</t>
+        </is>
+      </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -8304,7 +8444,7 @@
       </c>
       <c r="AA21" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 25. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про пирамиду Хеопса и записки. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 25. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про пирамиду Хеопса и записки. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -9435,7 +9575,11 @@
           <t>играет на дудочке</t>
         </is>
       </c>
-      <c r="M31" s="7" t="inlineStr"/>
+      <c r="M31" s="7" t="inlineStr">
+        <is>
+          <t>будит жителей</t>
+        </is>
+      </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -9496,7 +9640,7 @@
       </c>
       <c r="AA31" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 15. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/15. женщина будит жителей.jpeg; не скопирован в app/static. Решение Виктора: женщина будит жителей — использовать как визуальный вопрос. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 15. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/15. женщина будит жителей.jpeg; не скопирован в app/static. Решение Виктора: женщина будит жителей — использовать как визуальный вопрос. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -9557,7 +9701,11 @@
           <t>продажа купальников</t>
         </is>
       </c>
-      <c r="M32" s="7" t="inlineStr"/>
+      <c r="M32" s="7" t="inlineStr">
+        <is>
+          <t>конкурс красоты</t>
+        </is>
+      </c>
       <c r="N32" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -9618,7 +9766,7 @@
       </c>
       <c r="AA32" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 16. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/16. конкурс красоты.png; не скопирован в app/static. Решение Виктора: конкурс красоты/лодыжки оставить только после замены картинки на чистый источник; текущая выглядит обработанной. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 16. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/16. конкурс красоты.png; не скопирован в app/static. Решение Виктора: конкурс красоты/лодыжки оставить только после замены картинки на чистый источник; текущая выглядит обработанной. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -9679,7 +9827,11 @@
           <t>поднимают груз</t>
         </is>
       </c>
-      <c r="M33" s="7" t="inlineStr"/>
+      <c r="M33" s="7" t="inlineStr">
+        <is>
+          <t>спят</t>
+        </is>
+      </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -9740,7 +9892,7 @@
       </c>
       <c r="AA33" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 17. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/17. Двухпенсовый подвес.jpg; не скопирован в app/static. Решение Виктора: двухпенсовый подвес / люди спят на верёвках — использовать как визуальный вопрос. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 17. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/17. Двухпенсовый подвес.jpg; не скопирован в app/static. Решение Виктора: двухпенсовый подвес / люди спят на верёвках — использовать как визуальный вопрос. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -9801,7 +9953,11 @@
           <t>выбирали невесту</t>
         </is>
       </c>
-      <c r="M34" s="7" t="inlineStr"/>
+      <c r="M34" s="7" t="inlineStr">
+        <is>
+          <t>лечили спину</t>
+        </is>
+      </c>
       <c r="N34" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -9862,7 +10018,7 @@
       </c>
       <c r="AA34" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 18. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/18. Медведь).png; не скопирован в app/static. Решение Виктора: медведь лечит спину — оставить, но нужен source check. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 18. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/18. Медведь).png; не скопирован в app/static. Решение Виктора: медведь лечит спину — оставить, но нужен source check. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -9923,7 +10079,11 @@
           <t>пудреница</t>
         </is>
       </c>
-      <c r="M35" s="7" t="inlineStr"/>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
+          <t>уксусница</t>
+        </is>
+      </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -9984,7 +10144,7 @@
       </c>
       <c r="AA35" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 19. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/19. Уксусница.jpg; не скопирован в app/static. Решение Виктора: уксусница / коробочка с резким запахом — использовать как визуальный/object question. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 19. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/19. Уксусница.jpg; не скопирован в app/static. Решение Виктора: уксусница / коробочка с резким запахом — использовать как визуальный/object question. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -10045,7 +10205,11 @@
           <t>массажер</t>
         </is>
       </c>
-      <c r="M36" s="7" t="inlineStr"/>
+      <c r="M36" s="7" t="inlineStr">
+        <is>
+          <t>фен</t>
+        </is>
+      </c>
       <c r="N36" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -10101,7 +10265,7 @@
       </c>
       <c r="AA36" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 20. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: предшественник фена с кипятком пока не финализировать; нужен источник/картинка. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 20. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: предшественник фена с кипятком пока не финализировать; нужен источник/картинка. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -10162,7 +10326,11 @@
           <t>извлекать занозу.</t>
         </is>
       </c>
-      <c r="M37" s="7" t="inlineStr"/>
+      <c r="M37" s="7" t="inlineStr">
+        <is>
+          <t>застегивать пуговицы</t>
+        </is>
+      </c>
       <c r="N37" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -10222,7 +10390,7 @@
       </c>
       <c r="AA37" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 21. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: застёгиватель пуговиц / buttonhook — использовать как визуальный/object question. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 21. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: застёгиватель пуговиц / buttonhook — использовать как визуальный/object question. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -10833,7 +11001,11 @@
       <c r="J43" s="7" t="inlineStr"/>
       <c r="K43" s="7" t="inlineStr"/>
       <c r="L43" s="7" t="inlineStr"/>
-      <c r="M43" s="7" t="inlineStr"/>
+      <c r="M43" s="7" t="inlineStr">
+        <is>
+          <t>микроволновая печь</t>
+        </is>
+      </c>
       <c r="N43" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -10895,7 +11067,7 @@
       </c>
       <c r="AA43" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 5. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Микроволновка.jpg; не скопирован в app/static. Решение Виктора: микроволновка / растаявшая конфета — использовать как визуальный вопрос. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 5. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Микроволновка.jpg; не скопирован в app/static. Решение Виктора: микроволновка / растаявшая конфета — использовать как визуальный вопрос. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>
@@ -11162,7 +11334,11 @@
       <c r="J46" s="7" t="inlineStr"/>
       <c r="K46" s="7" t="inlineStr"/>
       <c r="L46" s="7" t="inlineStr"/>
-      <c r="M46" s="7" t="inlineStr"/>
+      <c r="M46" s="7" t="inlineStr">
+        <is>
+          <t>точное время</t>
+        </is>
+      </c>
       <c r="N46" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -11224,7 +11400,7 @@
       </c>
       <c r="AA46" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 8. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Продавщица времени.jpg; не скопирован в app/static. Решение Виктора: выбрать лучший вариант между Время.jpg и Продавщица времени.jpg после просмотра. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 8. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Продавщица времени.jpg; не скопирован в app/static. Решение Виктора: выбрать лучший вариант между Время.jpg и Продавщица времени.jpg после просмотра. Правильный ответ ещё нужно подтвердить/заполнить. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply remaining question bank v2 decisions
</commit_message>
<xml_diff>
--- a/docs/question_bank_v2/question_bank_v2_authoring_draft.xlsx
+++ b/docs/question_bank_v2/question_bank_v2_authoring_draft.xlsx
@@ -801,7 +801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X45"/>
+  <dimension ref="A1:X44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -954,11 +954,11 @@
     </row>
     <row r="2" ht="95" customHeight="1">
       <c r="A2" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q001</t>
+          <t>v2_edited_q002</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>В белорусской столице Минске установлен памятник картошке.</t>
+          <t>В 17 веке в Канаде вместо обычных денег расплачивались игральными картами</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
@@ -988,10 +988,14 @@
       </c>
       <c r="H2" s="7" t="n"/>
       <c r="I2" s="7" t="n"/>
-      <c r="J2" s="9" t="n"/>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K2" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr">
@@ -1001,7 +1005,7 @@
       </c>
       <c r="M2" s="11" t="inlineStr">
         <is>
-          <t>v2_edited_potato_monument</t>
+          <t>v2_edited_playing_card_money</t>
         </is>
       </c>
       <c r="N2" s="11" t="inlineStr"/>
@@ -1022,7 +1026,8 @@
       </c>
       <c r="R2" s="7" t="inlineStr">
         <is>
-          <t>Медиа из source_docs: проверить файл в source_docs.</t>
+          <t>(В одной из провинций закончились деньги, тогда интендант нарезал на кусочки игральные карты, подписал их и заверил печатью.)
+Медиа из source_docs: проверить файл в source_docs.</t>
         </is>
       </c>
       <c r="S2" s="9" t="inlineStr">
@@ -1037,7 +1042,7 @@
       </c>
       <c r="U2" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 6. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 7. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V2" s="9" t="inlineStr">
@@ -1054,11 +1059,11 @@
     </row>
     <row r="3" ht="95" customHeight="1">
       <c r="A3" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q002</t>
+          <t>v2_edited_q003</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
@@ -1073,7 +1078,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>В 17 веке в Канаде вместо обычных денег расплачивались игральными картами</t>
+          <t>В Польше Винни-Пуха называют Кубусь Пухатек</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -1098,25 +1103,21 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="M3" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_playing_card_money</t>
-        </is>
-      </c>
-      <c r="N3" s="11" t="inlineStr"/>
-      <c r="O3" s="11" t="inlineStr">
-        <is>
-          <t>needs_mapping</t>
-        </is>
-      </c>
-      <c r="P3" s="10" t="inlineStr">
-        <is>
-          <t>with_question</t>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr"/>
+      <c r="N3" s="7" t="inlineStr"/>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="P3" s="9" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
       <c r="Q3" s="7" t="inlineStr">
@@ -1126,8 +1127,7 @@
       </c>
       <c r="R3" s="7" t="inlineStr">
         <is>
-          <t>(В одной из провинций закончились деньги, тогда интендант нарезал на кусочки игральные карты, подписал их и заверил печатью.)
-Медиа из source_docs: проверить файл в source_docs.</t>
+          <t>(А живет от в Хатке Пухатке)</t>
         </is>
       </c>
       <c r="S3" s="9" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="U3" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 7. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 8. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V3" s="9" t="inlineStr">
@@ -1159,11 +1159,11 @@
     </row>
     <row r="4" ht="95" customHeight="1">
       <c r="A4" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q003</t>
+          <t>v2_edited_q004</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>В Польше Винни-Пуха называют Кубусь Пухатек</t>
+          <t>Курица проглатывает камешки, чтобы восполнить в организме недостающие минералы</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -1195,7 +1195,7 @@
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="9" t="inlineStr">
         <is>
-          <t>правда</t>
+          <t>ложь</t>
         </is>
       </c>
       <c r="K4" s="21" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="R4" s="7" t="inlineStr">
         <is>
-          <t>(А живет от в Хатке Пухатке)</t>
+          <t>(Камешки они проглатывают, но с другой целью. Они служат в желудке жерновами.)</t>
         </is>
       </c>
       <c r="S4" s="9" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="U4" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 8. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 9. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V4" s="9" t="inlineStr">
@@ -1259,11 +1259,11 @@
     </row>
     <row r="5" ht="95" customHeight="1">
       <c r="A5" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q004</t>
+          <t>v2_edited_q005</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Курица проглатывает камешки, чтобы восполнить в организме недостающие минералы</t>
+          <t>Матросы французского флота работали в условиях низких потолков на палубах кораблей. Помпоны на головных уборах служили для чистки потолков.</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="R5" s="7" t="inlineStr">
         <is>
-          <t>(Камешки они проглатывают, но с другой целью. Они служат в желудке жерновами.)</t>
+          <t>(Помпоны были для безопасности и смягчали возможный удар).</t>
         </is>
       </c>
       <c r="S5" s="9" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 9. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 10. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V5" s="9" t="inlineStr">
@@ -1359,11 +1359,11 @@
     </row>
     <row r="6" ht="95" customHeight="1">
       <c r="A6" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q005</t>
+          <t>v2_edited_q006</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Матросы французского флота работали в условиях низких потолков на палубах кораблей. Помпоны на головных уборах служили для чистки потолков.</t>
+          <t>Первоначально Google назывался BackRub.</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -1395,39 +1395,48 @@
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="9" t="inlineStr">
         <is>
-          <t>ложь</t>
-        </is>
-      </c>
-      <c r="K6" s="21" t="inlineStr">
+          <t>правда</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="L6" s="9" t="inlineStr">
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_backrub</t>
+        </is>
+      </c>
+      <c r="N6" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_backrub.jpg</t>
+        </is>
+      </c>
+      <c r="O6" s="11" t="inlineStr">
+        <is>
+          <t>source_available_unverified</t>
+        </is>
+      </c>
+      <c r="P6" s="10" t="inlineStr">
+        <is>
+          <t>after_answer</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="M6" s="7" t="inlineStr"/>
-      <c r="N6" s="7" t="inlineStr"/>
-      <c r="O6" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="P6" s="9" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="Q6" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
       <c r="R6" s="7" t="inlineStr">
         <is>
-          <t>(Помпоны были для безопасности и смягчали возможный удар).</t>
+          <t>(Да, в 1996 году студенты Стэнфордского университета Ларри Пейдж и Сергей Брин приступили к работе над поисковой системой, которую назвали BackRub (дословно это означает «массаж спины»). Фото «BackRub».
+Медиа из source_docs: BackRub.jpg.</t>
         </is>
       </c>
       <c r="S6" s="9" t="inlineStr">
@@ -1435,14 +1444,14 @@
           <t>easy</t>
         </is>
       </c>
-      <c r="T6" s="12" t="inlineStr">
-        <is>
-          <t>needs_review</t>
+      <c r="T6" s="10" t="inlineStr">
+        <is>
+          <t>needs_media</t>
         </is>
       </c>
       <c r="U6" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 10. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 11. Аудит action=keep. answer_type=true_false. risk_flags=needs_media, brand_fact_check. Исходный asset есть в docs/question_bank_v2/source_docs/BackRub.jpg; не скопирован в app/static. Решение Виктора: BackRub.jpg использовать как reveal/support image для вопроса про Google BackRub.</t>
         </is>
       </c>
       <c r="V6" s="9" t="inlineStr">
@@ -1459,11 +1468,11 @@
     </row>
     <row r="7" ht="95" customHeight="1">
       <c r="A7" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q006</t>
+          <t>v2_edited_q007</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -1478,7 +1487,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Первоначально Google назывался BackRub.</t>
+          <t>На персидском языке дворец называют сараем</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -1498,34 +1507,26 @@
           <t>правда</t>
         </is>
       </c>
-      <c r="K7" s="9" t="inlineStr">
+      <c r="K7" s="21" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="L7" s="10" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="M7" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_backrub</t>
-        </is>
-      </c>
-      <c r="N7" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_backrub.jpg</t>
-        </is>
-      </c>
-      <c r="O7" s="11" t="inlineStr">
-        <is>
-          <t>source_available_unverified</t>
-        </is>
-      </c>
-      <c r="P7" s="10" t="inlineStr">
-        <is>
-          <t>after_answer</t>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr"/>
+      <c r="N7" s="7" t="inlineStr"/>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
@@ -1535,8 +1536,7 @@
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>(Да, в 1996 году студенты Стэнфордского университета Ларри Пейдж и Сергей Брин приступили к работе над поисковой системой, которую назвали BackRub (дословно это означает «массаж спины»). Фото «BackRub».
-Медиа из source_docs: BackRub.jpg.</t>
+          <t>Слово “сарай” восходит к персидскому/иранскому слову со значением дворец, дом, помещение; формулировку лучше смягчить.</t>
         </is>
       </c>
       <c r="S7" s="9" t="inlineStr">
@@ -1544,14 +1544,14 @@
           <t>easy</t>
         </is>
       </c>
-      <c r="T7" s="10" t="inlineStr">
-        <is>
-          <t>needs_media</t>
+      <c r="T7" s="12" t="inlineStr">
+        <is>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 11. Аудит action=keep. answer_type=true_false. risk_flags=needs_media, brand_fact_check. Исходный asset есть в docs/question_bank_v2/source_docs/BackRub.jpg; не скопирован в app/static. Решение Виктора: BackRub.jpg использовать как reveal/support image для вопроса про Google BackRub.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 12. Аудит action=keep. answer_type=true_false. | Ответ заполнен по решению Виктора; смягчить формулировку перед импортом.</t>
         </is>
       </c>
       <c r="V7" s="9" t="inlineStr">
@@ -1568,11 +1568,11 @@
     </row>
     <row r="8" ht="95" customHeight="1">
       <c r="A8" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q007</t>
+          <t>v2_edited_q008</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>На персидском языке дворец называют сараем</t>
+          <t>У игры «Монополия» есть специальная горячая линия для урегулирования семейных конфликтов из-за споров о покупке недвижимости и траты денег?</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -1602,10 +1602,14 @@
       </c>
       <c r="H8" s="7" t="n"/>
       <c r="I8" s="7" t="n"/>
-      <c r="J8" s="9" t="n"/>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K8" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L8" s="9" t="inlineStr">
@@ -1630,7 +1634,11 @@
           <t>нет</t>
         </is>
       </c>
-      <c r="R8" s="7" t="n"/>
+      <c r="R8" s="7" t="inlineStr">
+        <is>
+          <t>Это не постоянная служба, а рождественская горячая линия/helpline Hasbro UK/Ireland для споров по Monopoly.</t>
+        </is>
+      </c>
       <c r="S8" s="9" t="inlineStr">
         <is>
           <t>easy</t>
@@ -1643,7 +1651,7 @@
       </c>
       <c r="U8" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 12. Аудит action=keep. answer_type=true_false.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 13. Аудит action=keep. answer_type=true_false. | Ответ заполнен по решению Виктора; проверить/смягчить формулировку перед импортом.</t>
         </is>
       </c>
       <c r="V8" s="9" t="inlineStr">
@@ -1660,11 +1668,11 @@
     </row>
     <row r="9" ht="95" customHeight="1">
       <c r="A9" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q008</t>
+          <t>v2_edited_q009</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -1679,7 +1687,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>У игры «Монополия» есть специальная горячая линия для урегулирования семейных конфликтов из-за споров о покупке недвижимости и траты денег?</t>
+          <t>Астероиды падают на Землю в среднем каждые 2 недели</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1694,10 +1702,14 @@
       </c>
       <c r="H9" s="7" t="n"/>
       <c r="I9" s="7" t="n"/>
-      <c r="J9" s="9" t="n"/>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="K9" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L9" s="9" t="inlineStr">
@@ -1722,7 +1734,11 @@
           <t>нет</t>
         </is>
       </c>
-      <c r="R9" s="7" t="n"/>
+      <c r="R9" s="7" t="inlineStr">
+        <is>
+          <t>(Астероиды не всегда большие и разрушительные. Небольшие астероиды (диаметр меньше метра) прилетают к нам в гости чаще чем теща или свекровь. И, как показывает статистика, несут с собой значительно меньше рисков._</t>
+        </is>
+      </c>
       <c r="S9" s="9" t="inlineStr">
         <is>
           <t>easy</t>
@@ -1735,7 +1751,7 @@
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 13. Аудит action=keep. answer_type=true_false.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 14. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про астероиды каждые 2 недели. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V9" s="9" t="inlineStr">
@@ -1752,11 +1768,11 @@
     </row>
     <row r="10" ht="95" customHeight="1">
       <c r="A10" s="9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q009</t>
+          <t>v2_edited_q011</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -1771,7 +1787,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Астероиды падают на Землю в среднем каждые 2 недели</t>
+          <t>Законодательство США допускало отправку детей по почте</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -1820,7 +1836,7 @@
       </c>
       <c r="R10" s="7" t="inlineStr">
         <is>
-          <t>(Астероиды не всегда большие и разрушительные. Небольшие астероиды (диаметр меньше метра) прилетают к нам в гости чаще чем теща или свекровь. И, как показывает статистика, несут с собой значительно меньше рисков._</t>
+          <t>( до 1913 года, когда был принят закон, запрещающий такие отправления).</t>
         </is>
       </c>
       <c r="S10" s="9" t="inlineStr">
@@ -1835,7 +1851,7 @@
       </c>
       <c r="U10" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 14. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про астероиды каждые 2 недели. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 16. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V10" s="9" t="inlineStr">
@@ -1852,11 +1868,11 @@
     </row>
     <row r="11" ht="95" customHeight="1">
       <c r="A11" s="9" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q011</t>
+          <t>v2_edited_q013</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -1871,7 +1887,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Законодательство США допускало отправку детей по почте</t>
+          <t>В фирменной пицце «Собрание» содержится перец халапеньо</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1918,11 +1934,7 @@
           <t>нет</t>
         </is>
       </c>
-      <c r="R11" s="7" t="inlineStr">
-        <is>
-          <t>( до 1913 года, когда был принят закон, запрещающий такие отправления).</t>
-        </is>
-      </c>
+      <c r="R11" s="7" t="n"/>
       <c r="S11" s="9" t="inlineStr">
         <is>
           <t>easy</t>
@@ -1935,7 +1947,7 @@
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 16. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 18. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить; внутренний факт подтверждён Виктором, в пицце Собрание есть халапеньо. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V11" s="9" t="inlineStr">
@@ -1952,11 +1964,11 @@
     </row>
     <row r="12" ht="95" customHeight="1">
       <c r="A12" s="9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q013</t>
+          <t>v2_edited_q014</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -1971,7 +1983,7 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>В фирменной пицце «Собрание» содержится перец халапеньо</t>
+          <t>Samsung тестирует смартфоны на прочность с помощью робота в форме ягодиц</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -2018,7 +2030,11 @@
           <t>нет</t>
         </is>
       </c>
-      <c r="R12" s="7" t="n"/>
+      <c r="R12" s="7" t="inlineStr">
+        <is>
+          <t>( Где чаще всего вы носите свой мобильный телефон? Ну, наверняка в заднем кармане брюк. Вот именно по этой причине компания Samsung сделали робота в форме ягодиц (он даже одет в джинсы!), который "сидит" на смартфонах, ...</t>
+        </is>
+      </c>
       <c r="S12" s="9" t="inlineStr">
         <is>
           <t>easy</t>
@@ -2031,7 +2047,7 @@
       </c>
       <c r="U12" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 18. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить; внутренний факт подтверждён Виктором, в пицце Собрание есть халапеньо. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 19. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V12" s="9" t="inlineStr">
@@ -2048,11 +2064,11 @@
     </row>
     <row r="13" ht="95" customHeight="1">
       <c r="A13" s="9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q014</t>
+          <t>v2_edited_q015</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -2067,7 +2083,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Samsung тестирует смартфоны на прочность с помощью робота в форме ягодиц</t>
+          <t>Маленький кармашек в джинсах предназначен для хранения презерватива.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -2084,7 +2100,7 @@
       <c r="I13" s="7" t="n"/>
       <c r="J13" s="9" t="inlineStr">
         <is>
-          <t>правда</t>
+          <t>ложь</t>
         </is>
       </c>
       <c r="K13" s="21" t="inlineStr">
@@ -2116,7 +2132,7 @@
       </c>
       <c r="R13" s="7" t="inlineStr">
         <is>
-          <t>( Где чаще всего вы носите свой мобильный телефон? Ну, наверняка в заднем кармане брюк. Вот именно по этой причине компания Samsung сделали робота в форме ягодиц (он даже одет в джинсы!), который "сидит" на смартфонах, ...</t>
+          <t>(Этот кармашек буквально назывался watch pocket (англ. «карман для часов»). Впервые его ввела компания Levi Strauss &amp; Co в 1800-х годах, чтобы ковбои могли безопасно хранить свои карманные часы на цепочке)</t>
         </is>
       </c>
       <c r="S13" s="9" t="inlineStr">
@@ -2131,7 +2147,7 @@
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 19. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 20. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V13" s="9" t="inlineStr">
@@ -2148,11 +2164,11 @@
     </row>
     <row r="14" ht="95" customHeight="1">
       <c r="A14" s="9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q015</t>
+          <t>v2_edited_q016</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -2167,7 +2183,7 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Маленький кармашек в джинсах предназначен для хранения презерватива.</t>
+          <t>Бананы растут вверх ногами</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -2184,7 +2200,7 @@
       <c r="I14" s="7" t="n"/>
       <c r="J14" s="9" t="inlineStr">
         <is>
-          <t>ложь</t>
+          <t>правда</t>
         </is>
       </c>
       <c r="K14" s="21" t="inlineStr">
@@ -2192,31 +2208,40 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L14" s="9" t="inlineStr">
+      <c r="L14" s="22" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="M14" s="19" t="inlineStr">
+        <is>
+          <t>v2_edited_banany</t>
+        </is>
+      </c>
+      <c r="N14" s="19" t="inlineStr">
+        <is>
+          <t>v2_edited_banany.jfif</t>
+        </is>
+      </c>
+      <c r="O14" s="19" t="inlineStr">
+        <is>
+          <t>needs_crop_or_replace</t>
+        </is>
+      </c>
+      <c r="P14" s="22" t="inlineStr">
+        <is>
+          <t>with_question</t>
+        </is>
+      </c>
+      <c r="Q14" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="M14" s="7" t="inlineStr"/>
-      <c r="N14" s="7" t="inlineStr"/>
-      <c r="O14" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="P14" s="9" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="Q14" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
       <c r="R14" s="7" t="inlineStr">
         <is>
-          <t>(Этот кармашек буквально назывался watch pocket (англ. «карман для часов»). Впервые его ввела компания Levi Strauss &amp; Co в 1800-х годах, чтобы ковбои могли безопасно хранить свои карманные часы на цепочке)</t>
+          <t>(Естественно, они растут из стеблей, но их нижняя часть на самом деле обращена вверх, к небу. По мере своего роста плоды поворачиваются к солнцу, образуя характерную дугообразную форму. (Фото Бананы)
+Медиа из source_docs: Бананы.jfif.</t>
         </is>
       </c>
       <c r="S14" s="9" t="inlineStr">
@@ -2224,14 +2249,14 @@
           <t>easy</t>
         </is>
       </c>
-      <c r="T14" s="12" t="inlineStr">
-        <is>
-          <t>needs_review</t>
+      <c r="T14" s="22" t="inlineStr">
+        <is>
+          <t>needs_crop_or_replace</t>
         </is>
       </c>
       <c r="U14" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 20. Аудит action=keep. answer_type=true_false. risk_flags=brand_fact_check. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 21. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Бананы.jfif; не скопирован в app/static. Решение Виктора: вопрос про бананы оставить как есть; картинку Бананы.jfif нужно кропнуть или заменить из-за чёрных полей. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V14" s="9" t="inlineStr">
@@ -2248,11 +2273,11 @@
     </row>
     <row r="15" ht="95" customHeight="1">
       <c r="A15" s="9" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q016</t>
+          <t>v2_edited_q018</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -2267,7 +2292,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Бананы растут вверх ногами</t>
+          <t>Черепахи могут дышать попой!</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -2292,29 +2317,21 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L15" s="22" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="M15" s="19" t="inlineStr">
-        <is>
-          <t>v2_edited_banany</t>
-        </is>
-      </c>
-      <c r="N15" s="19" t="inlineStr">
-        <is>
-          <t>v2_edited_banany.jfif</t>
-        </is>
-      </c>
-      <c r="O15" s="19" t="inlineStr">
-        <is>
-          <t>needs_crop_or_replace</t>
-        </is>
-      </c>
-      <c r="P15" s="22" t="inlineStr">
-        <is>
-          <t>with_question</t>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr"/>
+      <c r="N15" s="7" t="inlineStr"/>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="P15" s="9" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
@@ -2324,8 +2341,7 @@
       </c>
       <c r="R15" s="7" t="inlineStr">
         <is>
-          <t>(Естественно, они растут из стеблей, но их нижняя часть на самом деле обращена вверх, к небу. По мере своего роста плоды поворачиваются к солнцу, образуя характерную дугообразную форму. (Фото Бананы)
-Медиа из source_docs: Бананы.jfif.</t>
+          <t>(Технический термин - клоакальное дыхание)</t>
         </is>
       </c>
       <c r="S15" s="9" t="inlineStr">
@@ -2333,14 +2349,14 @@
           <t>easy</t>
         </is>
       </c>
-      <c r="T15" s="22" t="inlineStr">
-        <is>
-          <t>needs_crop_or_replace</t>
+      <c r="T15" s="12" t="inlineStr">
+        <is>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 21. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Бананы.jfif; не скопирован в app/static. Решение Виктора: вопрос про бананы оставить как есть; картинку Бананы.jfif нужно кропнуть или заменить из-за чёрных полей. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 23. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про черепах и клоакальное дыхание. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V15" s="9" t="inlineStr">
@@ -2357,11 +2373,11 @@
     </row>
     <row r="16" ht="95" customHeight="1">
       <c r="A16" s="9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q018</t>
+          <t>v2_edited_q019</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -2376,7 +2392,7 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Черепахи могут дышать попой!</t>
+          <t>Самолетный черный ящик имеет оранжевый цвет</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -2425,7 +2441,7 @@
       </c>
       <c r="R16" s="7" t="inlineStr">
         <is>
-          <t>(Технический термин - клоакальное дыхание)</t>
+          <t>(Это чтобы его легче было искать)</t>
         </is>
       </c>
       <c r="S16" s="9" t="inlineStr">
@@ -2440,7 +2456,7 @@
       </c>
       <c r="U16" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 23. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про черепах и клоакальное дыхание. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 24. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V16" s="9" t="inlineStr">
@@ -2457,11 +2473,11 @@
     </row>
     <row r="17" ht="95" customHeight="1">
       <c r="A17" s="9" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q019</t>
+          <t>v2_edited_q020</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -2476,7 +2492,7 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Самолетный черный ящик имеет оранжевый цвет</t>
+          <t>У туристов есть традиция оставлять друг другу записки между плит в пирамиде Хеопса</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -2493,7 +2509,7 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>правда</t>
+          <t>ложь</t>
         </is>
       </c>
       <c r="K17" s="21" t="inlineStr">
@@ -2525,7 +2541,7 @@
       </c>
       <c r="R17" s="7" t="inlineStr">
         <is>
-          <t>(Это чтобы его легче было искать)</t>
+          <t>(Между плитами (блоками) пирамиды Хеопса наблюдается чрезвычайно плотная подгонка, при которой зазор составляет всего около 0,5 миллиметра. Это означает, что в место стыка между двумя камнями невозможно протиснуть даже ...</t>
         </is>
       </c>
       <c r="S17" s="9" t="inlineStr">
@@ -2540,7 +2556,7 @@
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 24. Аудит action=keep. answer_type=true_false. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 25. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про пирамиду Хеопса и записки. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V17" s="9" t="inlineStr">
@@ -2557,16 +2573,16 @@
     </row>
     <row r="18" ht="95" customHeight="1">
       <c r="A18" s="9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q020</t>
+          <t>v2_edited_q021</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>v2_warmup_oath</t>
+          <t>v2_stories_tricks</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -2576,27 +2592,35 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>У туристов есть традиция оставлять друг другу записки между плит в пирамиде Хеопса</t>
+          <t>В кинофильме «Операция Ы» Трус, Бывалый и Балбес выступают в роли последователей известного русского хирурга Николая Пирогова. Как называется медицинское средство, которое они используют?</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>правда</t>
+          <t>спирт</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>ложь</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="n"/>
+          <t>хлороформ</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>пеницилин</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>бинты</t>
+        </is>
+      </c>
       <c r="J18" s="9" t="inlineStr">
         <is>
-          <t>ложь</t>
-        </is>
-      </c>
-      <c r="K18" s="21" t="inlineStr">
+          <t>хлороформ</t>
+        </is>
+      </c>
+      <c r="K18" s="9" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -2623,14 +2647,10 @@
           <t>нет</t>
         </is>
       </c>
-      <c r="R18" s="7" t="inlineStr">
-        <is>
-          <t>(Между плитами (блоками) пирамиды Хеопса наблюдается чрезвычайно плотная подгонка, при которой зазор составляет всего около 0,5 миллиметра. Это означает, что в место стыка между двумя камнями невозможно протиснуть даже ...</t>
-        </is>
-      </c>
+      <c r="R18" s="7" t="n"/>
       <c r="S18" s="9" t="inlineStr">
         <is>
-          <t>easy</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="T18" s="12" t="inlineStr">
@@ -2640,7 +2660,7 @@
       </c>
       <c r="U18" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 25. Аудит action=keep. answer_type=true_false. Решение Виктора: оставить как есть про пирамиду Хеопса и записки. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 6. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — хлороформ.</t>
         </is>
       </c>
       <c r="V18" s="9" t="inlineStr">
@@ -2657,16 +2677,16 @@
     </row>
     <row r="19" ht="95" customHeight="1">
       <c r="A19" s="9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q021</t>
+          <t>v2_edited_q022</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>v2_stories_tricks</t>
+          <t>v2_signs_objects</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -2676,32 +2696,32 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>В кинофильме «Операция Ы» Трус, Бывалый и Балбес выступают в роли последователей известного русского хирурга Николая Пирогова. Как называется медицинское средство, которое они используют?</t>
+          <t>Предприниматель Хироки Тэраи открыл необычный дворец для церемоний. Какие события там отмечали?</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>спирт</t>
+          <t>свадьбы</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>хлороформ</t>
+          <t>разводы</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>пеницилин</t>
+          <t>рождение</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>бинты</t>
+          <t>смерти</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>хлороформ</t>
+          <t>разводы</t>
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr">
@@ -2744,7 +2764,7 @@
       </c>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 6. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — хлороформ.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 7. Аудит action=rewrite. answer_type=multiple_choice. risk_flags=adult_or_dark_tone_review. Решение Виктора: оставить; правильный ответ — разводы.</t>
         </is>
       </c>
       <c r="V19" s="9" t="inlineStr">
@@ -2761,16 +2781,16 @@
     </row>
     <row r="20" ht="95" customHeight="1">
       <c r="A20" s="9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q022</t>
+          <t>v2_edited_q023</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>v2_signs_objects</t>
+          <t>v2_stories_tricks</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -2780,32 +2800,32 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Предприниматель Хироки Тэраи открыл необычный дворец для церемоний. Какие события там отмечали?</t>
+          <t>Иоанна Хмелевская считала, если дама перешагнула отметку 90, мужчина вправе кое-чего себе позволить не делать. В чем измеряется это самое 90?</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>свадьбы</t>
+          <t>в сантиметрах</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>разводы</t>
+          <t>годах</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>рождение</t>
+          <t>килограммах</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>смерти</t>
+          <t>километрах</t>
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr">
         <is>
-          <t>разводы</t>
+          <t>килограммы</t>
         </is>
       </c>
       <c r="K20" s="9" t="inlineStr">
@@ -2835,20 +2855,24 @@
           <t>нет</t>
         </is>
       </c>
-      <c r="R20" s="7" t="n"/>
+      <c r="R20" s="7" t="inlineStr">
+        <is>
+          <t>(Иоанна Хмелевская считала, что настоящий мужчина должен, помимо прочего, носить женщину на руках, но не слишком часто. При этом, если женщина преодолела планку в 90 килограммов, то, по мнению Хмелевской, мужчина вправе...</t>
+        </is>
+      </c>
       <c r="S20" s="9" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="T20" s="12" t="inlineStr">
-        <is>
-          <t>needs_review</t>
+      <c r="T20" s="21" t="inlineStr">
+        <is>
+          <t>needs_source_check</t>
         </is>
       </c>
       <c r="U20" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 7. Аудит action=rewrite. answer_type=multiple_choice. risk_flags=adult_or_dark_tone_review. Решение Виктора: оставить; правильный ответ — разводы.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 8. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — килограммы; нужен первоисточник/проверка цитаты.</t>
         </is>
       </c>
       <c r="V20" s="9" t="inlineStr">
@@ -2865,16 +2889,16 @@
     </row>
     <row r="21" ht="95" customHeight="1">
       <c r="A21" s="9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q023</t>
+          <t>v2_edited_q024</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>v2_stories_tricks</t>
+          <t>v2_signs_objects</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -2884,32 +2908,32 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Иоанна Хмелевская считала, если дама перешагнула отметку 90, мужчина вправе кое-чего себе позволить не делать. В чем измеряется это самое 90?</t>
+          <t>Однажды Джон Шепард-Барон кое-куда опоздал и не смог сделать важную для него вещь. После этого он изобрел это:</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>в сантиметрах</t>
+          <t>камеру хранения</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>годах</t>
+          <t>паркомат</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>килограммах</t>
+          <t>банкомат</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>километрах</t>
+          <t>кодовый замок</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>килограммы</t>
+          <t>банкомат</t>
         </is>
       </c>
       <c r="K21" s="9" t="inlineStr">
@@ -2941,7 +2965,7 @@
       </c>
       <c r="R21" s="7" t="inlineStr">
         <is>
-          <t>(Иоанна Хмелевская считала, что настоящий мужчина должен, помимо прочего, носить женщину на руках, но не слишком часто. При этом, если женщина преодолела планку в 90 килограммов, то, по мнению Хмелевской, мужчина вправе...</t>
+          <t>(На него повлияло то, что однажды он опоздал в банк и не смог снять деньги после закрытия)</t>
         </is>
       </c>
       <c r="S21" s="9" t="inlineStr">
@@ -2949,14 +2973,14 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="T21" s="21" t="inlineStr">
-        <is>
-          <t>needs_source_check</t>
+      <c r="T21" s="12" t="inlineStr">
+        <is>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 8. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — килограммы; нужен первоисточник/проверка цитаты.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 9. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — банкомат.</t>
         </is>
       </c>
       <c r="V21" s="9" t="inlineStr">
@@ -2973,16 +2997,16 @@
     </row>
     <row r="22" ht="95" customHeight="1">
       <c r="A22" s="9" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q024</t>
+          <t>v2_edited_q025</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>v2_signs_objects</t>
+          <t>v2_stories_tricks</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -2992,32 +3016,32 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Однажды Джон Шепард-Барон кое-куда опоздал и не смог сделать важную для него вещь. После этого он изобрел это:</t>
+          <t>Представим, что вы живете в Дании, вам исполнилось 25 лет, и тут родня начинает посыпать вас корицей. Что это значит?</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>камеру хранения</t>
+          <t>вы закончили ВУЗ</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>паркомат</t>
+          <t>У вас первая зарплата</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>банкомат</t>
+          <t>у вас нет второй половинки</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>кодовый замок</t>
+          <t>родня готовит шарлотку</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr">
         <is>
-          <t>банкомат</t>
+          <t>нет второй половинки</t>
         </is>
       </c>
       <c r="K22" s="9" t="inlineStr">
@@ -3049,7 +3073,7 @@
       </c>
       <c r="R22" s="7" t="inlineStr">
         <is>
-          <t>(На него повлияло то, что однажды он опоздал в банк и не смог снять деньги после закрытия)</t>
+          <t>(По легенде, традиция зародилась в XVI веке и связана с торговцами специями. Они много путешествовали, не задерживаясь на одном месте надолго, поэтому не успевали создать семью. Чтобы привлечь внимание потенциальных пар...</t>
         </is>
       </c>
       <c r="S22" s="9" t="inlineStr">
@@ -3064,7 +3088,7 @@
       </c>
       <c r="U22" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 9. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — банкомат.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 10. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — нет второй половинки.</t>
         </is>
       </c>
       <c r="V22" s="9" t="inlineStr">
@@ -3081,16 +3105,16 @@
     </row>
     <row r="23" ht="95" customHeight="1">
       <c r="A23" s="9" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q025</t>
+          <t>v2_edited_q026</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>v2_stories_tricks</t>
+          <t>v2_signs_objects</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -3100,32 +3124,32 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Представим, что вы живете в Дании, вам исполнилось 25 лет, и тут родня начинает посыпать вас корицей. Что это значит?</t>
+          <t>Какое из этих блюд названо по имени повара?</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>вы закончили ВУЗ</t>
+          <t>Яйца «Бенедикт»</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>У вас первая зарплата</t>
+          <t>Салат «Цезарь»</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>у вас нет второй половинки</t>
+          <t>Торт «Наполеон»</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>родня готовит шарлотку</t>
+          <t>Бефстроганов</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>нет второй половинки</t>
+          <t>салат Цезарь</t>
         </is>
       </c>
       <c r="K23" s="9" t="inlineStr">
@@ -3157,7 +3181,7 @@
       </c>
       <c r="R23" s="7" t="inlineStr">
         <is>
-          <t>(По легенде, традиция зародилась в XVI веке и связана с торговцами специями. Они много путешествовали, не задерживаясь на одном месте надолго, поэтому не успевали создать семью. Чтобы привлечь внимание потенциальных пар...</t>
+          <t>(Цезарь Кардини — американский повар итальянского происхождения, которому приписывают изобретение салата «Цезарь». Все остальные блюда названы в честь известных людей, но не поваров).</t>
         </is>
       </c>
       <c r="S23" s="9" t="inlineStr">
@@ -3172,7 +3196,7 @@
       </c>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 10. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — нет второй половинки.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 11. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — салат Цезарь.</t>
         </is>
       </c>
       <c r="V23" s="9" t="inlineStr">
@@ -3189,16 +3213,16 @@
     </row>
     <row r="24" ht="95" customHeight="1">
       <c r="A24" s="9" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q026</t>
+          <t>v2_edited_q027</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>v2_signs_objects</t>
+          <t>v2_stories_tricks</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -3208,32 +3232,32 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Какое из этих блюд названо по имени повара?</t>
+          <t>У кого из этих животных самый длинный язык?</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>Яйца «Бенедикт»</t>
+          <t>собака</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Салат «Цезарь»</t>
+          <t>жираф</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>Торт «Наполеон»</t>
+          <t>муравьед</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>Бефстроганов</t>
+          <t>слон</t>
         </is>
       </c>
       <c r="J24" s="9" t="inlineStr">
         <is>
-          <t>салат Цезарь</t>
+          <t>муравьед</t>
         </is>
       </c>
       <c r="K24" s="9" t="inlineStr">
@@ -3263,11 +3287,7 @@
           <t>нет</t>
         </is>
       </c>
-      <c r="R24" s="7" t="inlineStr">
-        <is>
-          <t>(Цезарь Кардини — американский повар итальянского происхождения, которому приписывают изобретение салата «Цезарь». Все остальные блюда названы в честь известных людей, но не поваров).</t>
-        </is>
-      </c>
+      <c r="R24" s="7" t="n"/>
       <c r="S24" s="9" t="inlineStr">
         <is>
           <t>medium</t>
@@ -3280,7 +3300,7 @@
       </c>
       <c r="U24" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 11. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — салат Цезарь.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 12. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — муравьед.</t>
         </is>
       </c>
       <c r="V24" s="9" t="inlineStr">
@@ -3297,99 +3317,104 @@
     </row>
     <row r="25" ht="95" customHeight="1">
       <c r="A25" s="9" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q027</t>
+          <t>v2_edited_q029</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>v2_stories_tricks</t>
+          <t>v2_signs_objects</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>plain_text</t>
+          <t>image_clue</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>У кого из этих животных самый длинный язык?</t>
+          <t>Благодаря чему Кеша из мультфильма «Блудный попугай» смог выбраться из клетки?</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>собака</t>
+          <t>пила</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>жираф</t>
+          <t>взрывное устройство</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>муравьед</t>
+          <t>карате</t>
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>слон</t>
-        </is>
-      </c>
-      <c r="J25" s="9" t="inlineStr">
-        <is>
-          <t>муравьед</t>
-        </is>
-      </c>
-      <c r="K25" s="9" t="inlineStr">
+          <t>просто отодвинул затвор</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="n"/>
+      <c r="K25" s="21" t="inlineStr">
+        <is>
+          <t>НЕТ — проверить видео/кадр</t>
+        </is>
+      </c>
+      <c r="L25" s="10" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="L25" s="9" t="inlineStr">
+      <c r="M25" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_parrot_cage</t>
+        </is>
+      </c>
+      <c r="N25" s="11" t="inlineStr"/>
+      <c r="O25" s="11" t="inlineStr">
+        <is>
+          <t>needs_mapping</t>
+        </is>
+      </c>
+      <c r="P25" s="10" t="inlineStr">
+        <is>
+          <t>with_question</t>
+        </is>
+      </c>
+      <c r="Q25" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="M25" s="7" t="inlineStr"/>
-      <c r="N25" s="7" t="inlineStr"/>
-      <c r="O25" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="P25" s="9" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="Q25" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="R25" s="7" t="n"/>
+      <c r="R25" s="7" t="inlineStr">
+        <is>
+          <t>(Тут нужна картинка на ответ или видео)
+Медиа из source_docs: проверить файл в source_docs. | Предварительный вариант по решению Виктора: D — просто отодвинул затвор. Финальный ответ ставить только после проверки кадра/видео.</t>
+        </is>
+      </c>
       <c r="S25" s="9" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="T25" s="12" t="inlineStr">
-        <is>
-          <t>needs_review</t>
+      <c r="T25" s="21" t="inlineStr">
+        <is>
+          <t>needs_video_check</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 12. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — муравьед.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 14. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. Решение Виктора: Кеша из Блудного попугая пока не финализировать; нужен точный кадр/видео. | Reserve. Проверить точный кадр/видео; до проверки финальный ответ не заполнять.</t>
         </is>
       </c>
       <c r="V25" s="9" t="inlineStr">
         <is>
-          <t>нет</t>
+          <t>да</t>
         </is>
       </c>
       <c r="W25" s="9" t="inlineStr">
@@ -3401,11 +3426,11 @@
     </row>
     <row r="26" ht="95" customHeight="1">
       <c r="A26" s="9" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q029</t>
+          <t>v2_edited_q030</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -3420,33 +3445,37 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Благодаря чему Кеша из мультфильма «Блудный попугай» смог выбраться из клетки?</t>
+          <t>На фото необычная женщина. Что она делает?</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>пила</t>
+          <t>отпугивает птиц</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>взрывное устройство</t>
+          <t>будит жителей</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>карате</t>
+          <t>курит</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>просто отодвинул затвор</t>
-        </is>
-      </c>
-      <c r="J26" s="9" t="n"/>
+          <t>играет на дудочке</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>будит жителей</t>
+        </is>
+      </c>
       <c r="K26" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>да</t>
         </is>
       </c>
       <c r="L26" s="10" t="inlineStr">
@@ -3456,13 +3485,17 @@
       </c>
       <c r="M26" s="11" t="inlineStr">
         <is>
-          <t>v2_edited_parrot_cage</t>
-        </is>
-      </c>
-      <c r="N26" s="11" t="inlineStr"/>
+          <t>v2_edited_knocker_up</t>
+        </is>
+      </c>
+      <c r="N26" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_knocker_up.jpeg</t>
+        </is>
+      </c>
       <c r="O26" s="11" t="inlineStr">
         <is>
-          <t>needs_mapping</t>
+          <t>source_available_unverified</t>
         </is>
       </c>
       <c r="P26" s="10" t="inlineStr">
@@ -3477,8 +3510,8 @@
       </c>
       <c r="R26" s="7" t="inlineStr">
         <is>
-          <t>(Тут нужна картинка на ответ или видео)
-Медиа из source_docs: проверить файл в source_docs.</t>
+          <t>(Она жила в Лондоне и имела необычную профессию — будильщица. Она использовала в своей работе плевательную трубку, попадая из неё горохом аж до четвёртого этажа.)
+Медиа из source_docs: 15. женщина будит жителей.jpeg.</t>
         </is>
       </c>
       <c r="S26" s="9" t="inlineStr">
@@ -3486,19 +3519,19 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="T26" s="21" t="inlineStr">
-        <is>
-          <t>needs_video_check</t>
+      <c r="T26" s="10" t="inlineStr">
+        <is>
+          <t>needs_media</t>
         </is>
       </c>
       <c r="U26" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 14. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. Решение Виктора: Кеша из Блудного попугая пока не финализировать; нужен точный кадр/видео.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 15. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/15. женщина будит жителей.jpeg; не скопирован в app/static. Решение Виктора: женщина будит жителей — использовать как визуальный вопрос. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V26" s="9" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>нет</t>
         </is>
       </c>
       <c r="W26" s="9" t="inlineStr">
@@ -3510,11 +3543,11 @@
     </row>
     <row r="27" ht="95" customHeight="1">
       <c r="A27" s="9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q030</t>
+          <t>v2_edited_q031</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
@@ -3529,32 +3562,32 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>На фото необычная женщина. Что она делает?</t>
+          <t>Что происходит на фото?</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>отпугивает птиц</t>
+          <t>Акция за феминизм</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>будит жителей</t>
+          <t>конкурс красоты</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>курит</t>
+          <t>девушки загорают</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>играет на дудочке</t>
+          <t>продажа купальников</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr">
         <is>
-          <t>будит жителей</t>
+          <t>конкурс красоты</t>
         </is>
       </c>
       <c r="K27" s="21" t="inlineStr">
@@ -3562,27 +3595,27 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L27" s="10" t="inlineStr">
+      <c r="L27" s="22" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="M27" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_knocker_up</t>
-        </is>
-      </c>
-      <c r="N27" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_knocker_up.jpeg</t>
-        </is>
-      </c>
-      <c r="O27" s="11" t="inlineStr">
-        <is>
-          <t>source_available_unverified</t>
-        </is>
-      </c>
-      <c r="P27" s="10" t="inlineStr">
+      <c r="M27" s="19" t="inlineStr">
+        <is>
+          <t>v2_edited_beauty_contest</t>
+        </is>
+      </c>
+      <c r="N27" s="19" t="inlineStr">
+        <is>
+          <t>v2_edited_beauty_contest.png</t>
+        </is>
+      </c>
+      <c r="O27" s="19" t="inlineStr">
+        <is>
+          <t>needs_replacement</t>
+        </is>
+      </c>
+      <c r="P27" s="22" t="inlineStr">
         <is>
           <t>with_question</t>
         </is>
@@ -3594,8 +3627,8 @@
       </c>
       <c r="R27" s="7" t="inlineStr">
         <is>
-          <t>(Она жила в Лондоне и имела необычную профессию — будильщица. Она использовала в своей работе плевательную трубку, попадая из неё горохом аж до четвёртого этажа.)
-Медиа из source_docs: 15. женщина будит жителей.jpeg.</t>
+          <t>(Это конкурс красоты женских лодыжек. Жюри просили закрыть лица участниц, чтобы обращать внимание только на ноги.)
+Медиа из source_docs: 16. конкурс красоты.png.</t>
         </is>
       </c>
       <c r="S27" s="9" t="inlineStr">
@@ -3603,14 +3636,14 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="T27" s="10" t="inlineStr">
-        <is>
-          <t>needs_media</t>
+      <c r="T27" s="22" t="inlineStr">
+        <is>
+          <t>needs_replacement</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 15. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/15. женщина будит жителей.jpeg; не скопирован в app/static. Решение Виктора: женщина будит жителей — использовать как визуальный вопрос. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 16. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/16. конкурс красоты.png; не скопирован в app/static. Решение Виктора: конкурс красоты/лодыжки оставить только после замены картинки на чистый источник; текущая выглядит обработанной. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V27" s="9" t="inlineStr">
@@ -3627,11 +3660,11 @@
     </row>
     <row r="28" ht="95" customHeight="1">
       <c r="A28" s="9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q031</t>
+          <t>v2_edited_q032</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
@@ -3646,32 +3679,32 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Что происходит на фото?</t>
+          <t>На снимке происходит что-то необычное. Что делают эти люди?</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Акция за феминизм</t>
+          <t>проверяют прочность веревки</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>конкурс красоты</t>
+          <t>лечат мигрень</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>девушки загорают</t>
+          <t>спят</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>продажа купальников</t>
+          <t>поднимают груз</t>
         </is>
       </c>
       <c r="J28" s="9" t="inlineStr">
         <is>
-          <t>конкурс красоты</t>
+          <t>спят</t>
         </is>
       </c>
       <c r="K28" s="21" t="inlineStr">
@@ -3679,27 +3712,27 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L28" s="22" t="inlineStr">
+      <c r="L28" s="10" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="M28" s="19" t="inlineStr">
-        <is>
-          <t>v2_edited_beauty_contest</t>
-        </is>
-      </c>
-      <c r="N28" s="19" t="inlineStr">
-        <is>
-          <t>v2_edited_beauty_contest.png</t>
-        </is>
-      </c>
-      <c r="O28" s="19" t="inlineStr">
-        <is>
-          <t>needs_replacement</t>
-        </is>
-      </c>
-      <c r="P28" s="22" t="inlineStr">
+      <c r="M28" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_two_penny_hangover</t>
+        </is>
+      </c>
+      <c r="N28" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_two_penny_hangover.jpg</t>
+        </is>
+      </c>
+      <c r="O28" s="11" t="inlineStr">
+        <is>
+          <t>source_available_unverified</t>
+        </is>
+      </c>
+      <c r="P28" s="10" t="inlineStr">
         <is>
           <t>with_question</t>
         </is>
@@ -3711,8 +3744,8 @@
       </c>
       <c r="R28" s="7" t="inlineStr">
         <is>
-          <t>(Это конкурс красоты женских лодыжек. Жюри просили закрыть лица участниц, чтобы обращать внимание только на ноги.)
-Медиа из source_docs: 16. конкурс красоты.png.</t>
+          <t>(Фото сделано в Лондоне, где люди спали на веревках. Удовольствие стоило 2 цента и получило название 2-х пенсовый подвес. Так спали бедные бездомные люди.Так спать гораздо лучше, чем просто лежать на голом полу. Часто п...
+Медиа из source_docs: 17. Двухпенсовый подвес.jpg.</t>
         </is>
       </c>
       <c r="S28" s="9" t="inlineStr">
@@ -3720,14 +3753,14 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="T28" s="22" t="inlineStr">
-        <is>
-          <t>needs_replacement</t>
+      <c r="T28" s="10" t="inlineStr">
+        <is>
+          <t>needs_media</t>
         </is>
       </c>
       <c r="U28" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 16. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/16. конкурс красоты.png; не скопирован в app/static. Решение Виктора: конкурс красоты/лодыжки оставить только после замены картинки на чистый источник; текущая выглядит обработанной. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 17. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/17. Двухпенсовый подвес.jpg; не скопирован в app/static. Решение Виктора: двухпенсовый подвес / люди спят на верёвках — использовать как визуальный вопрос. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V28" s="9" t="inlineStr">
@@ -3744,11 +3777,11 @@
     </row>
     <row r="29" ht="95" customHeight="1">
       <c r="A29" s="9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q032</t>
+          <t>v2_edited_q033</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
@@ -3763,32 +3796,32 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>На снимке происходит что-то необычное. Что делают эти люди?</t>
+          <t>Под фото стерлась надпись. В Румынии так:</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>проверяют прочность веревки</t>
+          <t>приручали медведя</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>лечат мигрень</t>
+          <t>лечили спину</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>спят</t>
+          <t>изгоняли духов</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>поднимают груз</t>
+          <t>выбирали невесту</t>
         </is>
       </c>
       <c r="J29" s="9" t="inlineStr">
         <is>
-          <t>спят</t>
+          <t>лечили спину</t>
         </is>
       </c>
       <c r="K29" s="21" t="inlineStr">
@@ -3796,27 +3829,27 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L29" s="10" t="inlineStr">
+      <c r="L29" s="21" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="M29" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_two_penny_hangover</t>
-        </is>
-      </c>
-      <c r="N29" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_two_penny_hangover.jpg</t>
-        </is>
-      </c>
-      <c r="O29" s="11" t="inlineStr">
-        <is>
-          <t>source_available_unverified</t>
-        </is>
-      </c>
-      <c r="P29" s="10" t="inlineStr">
+      <c r="M29" s="20" t="inlineStr">
+        <is>
+          <t>v2_edited_bear_back</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="inlineStr">
+        <is>
+          <t>v2_edited_bear_back.png</t>
+        </is>
+      </c>
+      <c r="O29" s="20" t="inlineStr">
+        <is>
+          <t>needs_source_check</t>
+        </is>
+      </c>
+      <c r="P29" s="21" t="inlineStr">
         <is>
           <t>with_question</t>
         </is>
@@ -3828,8 +3861,8 @@
       </c>
       <c r="R29" s="7" t="inlineStr">
         <is>
-          <t>(Фото сделано в Лондоне, где люди спали на веревках. Удовольствие стоило 2 цента и получило название 2-х пенсовый подвес. Так спали бедные бездомные люди.Так спать гораздо лучше, чем просто лежать на голом полу. Часто п...
-Медиа из source_docs: 17. Двухпенсовый подвес.jpg.</t>
+          <t>(В 1946 году румынские цыгане так лечили спину. Урсары – дрессировщики медведей – таким образом вправляли позвонки или выравнивали осанку.)
+Медиа из source_docs: 18. Медведь).png.</t>
         </is>
       </c>
       <c r="S29" s="9" t="inlineStr">
@@ -3837,14 +3870,14 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="T29" s="10" t="inlineStr">
-        <is>
-          <t>needs_media</t>
+      <c r="T29" s="21" t="inlineStr">
+        <is>
+          <t>needs_source_check</t>
         </is>
       </c>
       <c r="U29" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 17. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/17. Двухпенсовый подвес.jpg; не скопирован в app/static. Решение Виктора: двухпенсовый подвес / люди спят на верёвках — использовать как визуальный вопрос. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 18. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/18. Медведь).png; не скопирован в app/static. Решение Виктора: медведь лечит спину — оставить, но нужен source check. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V29" s="9" t="inlineStr">
@@ -3861,11 +3894,11 @@
     </row>
     <row r="30" ht="95" customHeight="1">
       <c r="A30" s="9" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q033</t>
+          <t>v2_edited_q034</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -3880,32 +3913,32 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Под фото стерлась надпись. В Румынии так:</t>
+          <t>Вы взяли в руку маленькую коробочку с резким запахом. Она использовалась для того, чтобы привести даму в чувства после обморока. Как называлась эта коробочка?</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>приручали медведя</t>
+          <t>уксусница</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>лечили спину</t>
+          <t>табакерка</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>изгоняли духов</t>
+          <t>перечница</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>выбирали невесту</t>
+          <t>пудреница</t>
         </is>
       </c>
       <c r="J30" s="9" t="inlineStr">
         <is>
-          <t>лечили спину</t>
+          <t>уксусница</t>
         </is>
       </c>
       <c r="K30" s="21" t="inlineStr">
@@ -3913,27 +3946,27 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L30" s="21" t="inlineStr">
+      <c r="L30" s="10" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="M30" s="20" t="inlineStr">
-        <is>
-          <t>v2_edited_bear_back</t>
-        </is>
-      </c>
-      <c r="N30" s="20" t="inlineStr">
-        <is>
-          <t>v2_edited_bear_back.png</t>
-        </is>
-      </c>
-      <c r="O30" s="20" t="inlineStr">
-        <is>
-          <t>needs_source_check</t>
-        </is>
-      </c>
-      <c r="P30" s="21" t="inlineStr">
+      <c r="M30" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_vinaigrette_box</t>
+        </is>
+      </c>
+      <c r="N30" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_vinaigrette_box.jpg</t>
+        </is>
+      </c>
+      <c r="O30" s="11" t="inlineStr">
+        <is>
+          <t>source_available_unverified</t>
+        </is>
+      </c>
+      <c r="P30" s="10" t="inlineStr">
         <is>
           <t>with_question</t>
         </is>
@@ -3945,8 +3978,8 @@
       </c>
       <c r="R30" s="7" t="inlineStr">
         <is>
-          <t>(В 1946 году румынские цыгане так лечили спину. Урсары – дрессировщики медведей – таким образом вправляли позвонки или выравнивали осанку.)
-Медиа из source_docs: 18. Медведь).png.</t>
+          <t>(В эти коробочки укладывали ватки, которые смачивались уксусом)
+Медиа из source_docs: 19. Уксусница.jpg.</t>
         </is>
       </c>
       <c r="S30" s="9" t="inlineStr">
@@ -3954,14 +3987,14 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="T30" s="21" t="inlineStr">
-        <is>
-          <t>needs_source_check</t>
+      <c r="T30" s="10" t="inlineStr">
+        <is>
+          <t>needs_media</t>
         </is>
       </c>
       <c r="U30" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 18. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/18. Медведь).png; не скопирован в app/static. Решение Виктора: медведь лечит спину — оставить, но нужен source check. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 19. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/19. Уксусница.jpg; не скопирован в app/static. Решение Виктора: уксусница / коробочка с резким запахом — использовать как визуальный/object question. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V30" s="9" t="inlineStr">
@@ -3978,51 +4011,51 @@
     </row>
     <row r="31" ht="95" customHeight="1">
       <c r="A31" s="9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q034</t>
+          <t>v2_edited_q035</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>v2_signs_objects</t>
+          <t>v2_stories_tricks</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>image_clue</t>
+          <t>plain_text</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Вы взяли в руку маленькую коробочку с резким запахом. Она использовалась для того, чтобы привести даму в чувства после обморока. Как называлась эта коробочка?</t>
+          <t>Эта вещь что-то напоминает. Туда можно залить воду. Что это?</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>уксусница</t>
+          <t>утюг</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>табакерка</t>
+          <t>фен</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>перечница</t>
+          <t>грелка</t>
         </is>
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>пудреница</t>
+          <t>массажер</t>
         </is>
       </c>
       <c r="J31" s="9" t="inlineStr">
         <is>
-          <t>уксусница</t>
+          <t>фен</t>
         </is>
       </c>
       <c r="K31" s="21" t="inlineStr">
@@ -4030,29 +4063,21 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L31" s="10" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="M31" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_vinaigrette_box</t>
-        </is>
-      </c>
-      <c r="N31" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_vinaigrette_box.jpg</t>
-        </is>
-      </c>
-      <c r="O31" s="11" t="inlineStr">
-        <is>
-          <t>source_available_unverified</t>
-        </is>
-      </c>
-      <c r="P31" s="10" t="inlineStr">
-        <is>
-          <t>with_question</t>
+      <c r="L31" s="9" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="inlineStr"/>
+      <c r="N31" s="7" t="inlineStr"/>
+      <c r="O31" s="7" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="P31" s="9" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
       <c r="Q31" s="7" t="inlineStr">
@@ -4062,8 +4087,7 @@
       </c>
       <c r="R31" s="7" t="inlineStr">
         <is>
-          <t>(В эти коробочки укладывали ватки, которые смачивались уксусом)
-Медиа из source_docs: 19. Уксусница.jpg.</t>
+          <t>(Это предшественник современного фена. Чтобы высушить волосы достаточно было налить в эту емкость кипяток)</t>
         </is>
       </c>
       <c r="S31" s="9" t="inlineStr">
@@ -4071,14 +4095,14 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="T31" s="10" t="inlineStr">
-        <is>
-          <t>needs_media</t>
+      <c r="T31" s="21" t="inlineStr">
+        <is>
+          <t>needs_source_check</t>
         </is>
       </c>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 19. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/19. Уксусница.jpg; не скопирован в app/static. Решение Виктора: уксусница / коробочка с резким запахом — использовать как визуальный/object question. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 20. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: предшественник фена с кипятком пока не финализировать; нужен источник/картинка. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V31" s="9" t="inlineStr">
@@ -4095,51 +4119,51 @@
     </row>
     <row r="32" ht="95" customHeight="1">
       <c r="A32" s="9" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q035</t>
+          <t>v2_edited_q036</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>v2_stories_tricks</t>
+          <t>v2_signs_objects</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>plain_text</t>
+          <t>image_clue</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>Эта вещь что-то напоминает. Туда можно залить воду. Что это?</t>
+          <t>Таир-батон или батонхук. Для кимоно оно вряд ли бы пригодилось. Для чего нужен этот предмет?</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>утюг</t>
+          <t>штопать одежду</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>фен</t>
+          <t>вышивать</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>грелка</t>
+          <t>застегивать пуговицы</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>массажер</t>
+          <t>извлекать занозу.</t>
         </is>
       </c>
       <c r="J32" s="9" t="inlineStr">
         <is>
-          <t>фен</t>
+          <t>застегивать пуговицы</t>
         </is>
       </c>
       <c r="K32" s="21" t="inlineStr">
@@ -4147,31 +4171,39 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L32" s="9" t="inlineStr">
+      <c r="L32" s="10" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="M32" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_buttonhook</t>
+        </is>
+      </c>
+      <c r="N32" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_buttonhook.jpg</t>
+        </is>
+      </c>
+      <c r="O32" s="11" t="inlineStr">
+        <is>
+          <t>source_available_unverified</t>
+        </is>
+      </c>
+      <c r="P32" s="10" t="inlineStr">
+        <is>
+          <t>with_question</t>
+        </is>
+      </c>
+      <c r="Q32" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="M32" s="7" t="inlineStr"/>
-      <c r="N32" s="7" t="inlineStr"/>
-      <c r="O32" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="P32" s="9" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="Q32" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
       <c r="R32" s="7" t="inlineStr">
         <is>
-          <t>(Это предшественник современного фена. Чтобы высушить волосы достаточно было налить в эту емкость кипяток)</t>
+          <t>(Застегивать пуговицы. Тогда молнии еще не были изобретены, использовались разные крючки. Миниатюрные для белья или большие для обуви.)</t>
         </is>
       </c>
       <c r="S32" s="9" t="inlineStr">
@@ -4179,14 +4211,14 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="T32" s="21" t="inlineStr">
-        <is>
-          <t>needs_source_check</t>
+      <c r="T32" s="10" t="inlineStr">
+        <is>
+          <t>needs_media</t>
         </is>
       </c>
       <c r="U32" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 20. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: предшественник фена с кипятком пока не финализировать; нужен источник/картинка. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 21. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: застёгиватель пуговиц / buttonhook — использовать как визуальный/object question. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V32" s="9" t="inlineStr">
@@ -4203,51 +4235,51 @@
     </row>
     <row r="33" ht="95" customHeight="1">
       <c r="A33" s="9" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q036</t>
+          <t>v2_edited_q037</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>v2_signs_objects</t>
+          <t>v2_reserve</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>image_clue</t>
+          <t>plain_text</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Таир-батон или батонхук. Для кимоно оно вряд ли бы пригодилось. Для чего нужен этот предмет?</t>
+          <t>Какой предмет гигиены был централизованно введен через армию?</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>штопать одежду</t>
+          <t>бритва</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>вышивать</t>
+          <t>зубная щетка</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>застегивать пуговицы</t>
+          <t>ушные палочки</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>извлекать занозу.</t>
+          <t>расческа</t>
         </is>
       </c>
       <c r="J33" s="9" t="inlineStr">
         <is>
-          <t>застегивать пуговицы</t>
+          <t>зубная щётка</t>
         </is>
       </c>
       <c r="K33" s="21" t="inlineStr">
@@ -4255,59 +4287,51 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L33" s="10" t="inlineStr">
+      <c r="L33" s="9" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M33" s="7" t="inlineStr"/>
+      <c r="N33" s="7" t="inlineStr"/>
+      <c r="O33" s="7" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="P33" s="9" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Q33" s="7" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="R33" s="7" t="inlineStr">
+        <is>
+          <t>Резервная строка: использовать только после редакторского отбора. | Армейская дисциплина и военные гигиенические практики сильно распространили регулярную чистку зубов; формулировку надо смягчить.</t>
+        </is>
+      </c>
+      <c r="S33" s="9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T33" s="21" t="inlineStr">
+        <is>
+          <t>needs_source_check</t>
+        </is>
+      </c>
+      <c r="U33" s="7" t="inlineStr">
+        <is>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 22. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: предмет гигиены через армию — reserve/source_check. | Reserve/source_check. Ответ заполнен по решению Виктора; смягчить формулировку и проверить источник.</t>
+        </is>
+      </c>
+      <c r="V33" s="9" t="inlineStr">
         <is>
           <t>да</t>
-        </is>
-      </c>
-      <c r="M33" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_buttonhook</t>
-        </is>
-      </c>
-      <c r="N33" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_buttonhook.jpg</t>
-        </is>
-      </c>
-      <c r="O33" s="11" t="inlineStr">
-        <is>
-          <t>source_available_unverified</t>
-        </is>
-      </c>
-      <c r="P33" s="10" t="inlineStr">
-        <is>
-          <t>with_question</t>
-        </is>
-      </c>
-      <c r="Q33" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="R33" s="7" t="inlineStr">
-        <is>
-          <t>(Застегивать пуговицы. Тогда молнии еще не были изобретены, использовались разные крючки. Миниатюрные для белья или большие для обуви.)</t>
-        </is>
-      </c>
-      <c r="S33" s="9" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="T33" s="10" t="inlineStr">
-        <is>
-          <t>needs_media</t>
-        </is>
-      </c>
-      <c r="U33" s="7" t="inlineStr">
-        <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 21. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: застёгиватель пуговиц / buttonhook — использовать как визуальный/object question. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
-        </is>
-      </c>
-      <c r="V33" s="9" t="inlineStr">
-        <is>
-          <t>нет</t>
         </is>
       </c>
       <c r="W33" s="9" t="inlineStr">
@@ -4319,11 +4343,11 @@
     </row>
     <row r="34" ht="95" customHeight="1">
       <c r="A34" s="9" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q037</t>
+          <t>v2_edited_q038</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -4338,33 +4362,37 @@
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Какой предмет гигиены был централизованно введен через армию?</t>
+          <t>Какая особенность была у первых электрических тостеров?</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>бритва</t>
+          <t>работали на монетках</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>зубная щетка</t>
+          <t>подрумянивали с одной стороны</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>ушные палочки</t>
+          <t>хлеб крутился на вертеле</t>
         </is>
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>расческа</t>
-        </is>
-      </c>
-      <c r="J34" s="9" t="n"/>
-      <c r="K34" s="21" t="inlineStr">
-        <is>
-          <t>НЕТ — заполнить/проверить</t>
+          <t>коптили</t>
+        </is>
+      </c>
+      <c r="J34" s="9" t="inlineStr">
+        <is>
+          <t>подрумянивали с одной стороны</t>
+        </is>
+      </c>
+      <c r="K34" s="9" t="inlineStr">
+        <is>
+          <t>да</t>
         </is>
       </c>
       <c r="L34" s="9" t="inlineStr">
@@ -4391,7 +4419,8 @@
       </c>
       <c r="R34" s="7" t="inlineStr">
         <is>
-          <t>Резервная строка: использовать только после редакторского отбора.</t>
+          <t>(Хлеб приходилось переворачивать – это было неудобно)
+Резервная строка: использовать только после редакторского отбора.</t>
         </is>
       </c>
       <c r="S34" s="9" t="inlineStr">
@@ -4399,14 +4428,14 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="T34" s="21" t="inlineStr">
-        <is>
-          <t>needs_source_check</t>
+      <c r="T34" s="12" t="inlineStr">
+        <is>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="U34" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 22. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: предмет гигиены через армию — reserve/source_check.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 23. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — подрумянивали с одной стороны.</t>
         </is>
       </c>
       <c r="V34" s="9" t="inlineStr">
@@ -4423,11 +4452,11 @@
     </row>
     <row r="35" ht="95" customHeight="1">
       <c r="A35" s="9" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q038</t>
+          <t>v2_edited_q039</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -4437,37 +4466,21 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>plain_text</t>
+          <t>duel_question</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Какая особенность была у первых электрических тостеров?</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>работали на монетках</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>подрумянивали с одной стороны</t>
-        </is>
-      </c>
-      <c r="H35" s="7" t="inlineStr">
-        <is>
-          <t>хлеб крутился на вертеле</t>
-        </is>
-      </c>
-      <c r="I35" s="7" t="inlineStr">
-        <is>
-          <t>коптили</t>
-        </is>
-      </c>
+          <t>В Африке этот деликатес называют «летающими креветками пустыни». Что это такое?</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="n"/>
+      <c r="G35" s="7" t="n"/>
+      <c r="H35" s="7" t="n"/>
+      <c r="I35" s="7" t="n"/>
       <c r="J35" s="9" t="inlineStr">
         <is>
-          <t>подрумянивали с одной стороны</t>
+          <t>саранча</t>
         </is>
       </c>
       <c r="K35" s="9" t="inlineStr">
@@ -4499,8 +4512,7 @@
       </c>
       <c r="R35" s="7" t="inlineStr">
         <is>
-          <t>(Хлеб приходилось переворачивать – это было неудобно)
-Резервная строка: использовать только после редакторского отбора.</t>
+          <t>Резервная строка: использовать только после редакторского отбора.</t>
         </is>
       </c>
       <c r="S35" s="9" t="inlineStr">
@@ -4515,7 +4527,7 @@
       </c>
       <c r="U35" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 23. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: оставить; правильный ответ — подрумянивали с одной стороны.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 1. Аудит action=reserve. answer_type=open_answer.</t>
         </is>
       </c>
       <c r="V35" s="9" t="inlineStr">
@@ -4532,11 +4544,11 @@
     </row>
     <row r="36" ht="95" customHeight="1">
       <c r="A36" s="9" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q039</t>
+          <t>v2_edited_q040</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -4546,12 +4558,12 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>duel_question</t>
+          <t>image_clue</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>В Африке этот деликатес называют «летающими креветками пустыни». Что это такое?</t>
+          <t>Согласно итальянской народной мудрости, салат должны готовить четыре повара:</t>
         </is>
       </c>
       <c r="F36" s="7" t="n"/>
@@ -4560,7 +4572,7 @@
       <c r="I36" s="7" t="n"/>
       <c r="J36" s="9" t="inlineStr">
         <is>
-          <t>саранча</t>
+          <t>Смешивать ингредиенты.</t>
         </is>
       </c>
       <c r="K36" s="9" t="inlineStr">
@@ -4568,31 +4580,37 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L36" s="9" t="inlineStr">
+      <c r="L36" s="10" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="M36" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_time_salad</t>
+        </is>
+      </c>
+      <c r="N36" s="11" t="inlineStr"/>
+      <c r="O36" s="11" t="inlineStr">
+        <is>
+          <t>needs_mapping</t>
+        </is>
+      </c>
+      <c r="P36" s="10" t="inlineStr">
+        <is>
+          <t>with_question</t>
+        </is>
+      </c>
+      <c r="Q36" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="M36" s="7" t="inlineStr"/>
-      <c r="N36" s="7" t="inlineStr"/>
-      <c r="O36" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="P36" s="9" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="Q36" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
       <c r="R36" s="7" t="inlineStr">
         <is>
-          <t>Резервная строка: использовать только после редакторского отбора.</t>
+          <t>скупой заправляет салат уксусом, философ добавляет в него соль, щедрый поливает его маслом. Что должен сделать четвертый повар-художник во время приготовления салата?
+Медиа из source_docs: Время.png.
+Резервная строка: использовать только после редакторского отбора.</t>
         </is>
       </c>
       <c r="S36" s="9" t="inlineStr">
@@ -4600,14 +4618,14 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="T36" s="12" t="inlineStr">
-        <is>
-          <t>needs_review</t>
+      <c r="T36" s="10" t="inlineStr">
+        <is>
+          <t>needs_media</t>
         </is>
       </c>
       <c r="U36" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 1. Аудит action=reserve. answer_type=open_answer.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 2. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Время.png; не скопирован в app/static.</t>
         </is>
       </c>
       <c r="V36" s="9" t="inlineStr">
@@ -4624,11 +4642,11 @@
     </row>
     <row r="37" ht="95" customHeight="1">
       <c r="A37" s="9" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q040</t>
+          <t>v2_edited_q041</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
@@ -4643,7 +4661,7 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Согласно итальянской народной мудрости, салат должны готовить четыре повара:</t>
+          <t>Перед вами рекламный плакат нового изобретения «Вы нажимаете на кнопку, мы делаем все остальное». В 2000 компания была лидером продаж. Что рекламировал данный плакат?</t>
         </is>
       </c>
       <c r="F37" s="7" t="n"/>
@@ -4652,7 +4670,7 @@
       <c r="I37" s="7" t="n"/>
       <c r="J37" s="9" t="inlineStr">
         <is>
-          <t>Смешивать ингредиенты.</t>
+          <t>фотокамеру</t>
         </is>
       </c>
       <c r="K37" s="9" t="inlineStr">
@@ -4667,13 +4685,17 @@
       </c>
       <c r="M37" s="11" t="inlineStr">
         <is>
-          <t>v2_edited_time_salad</t>
-        </is>
-      </c>
-      <c r="N37" s="11" t="inlineStr"/>
+          <t>v2_edited_kodak_2</t>
+        </is>
+      </c>
+      <c r="N37" s="11" t="inlineStr">
+        <is>
+          <t>v2_edited_kodak_2.jpg</t>
+        </is>
+      </c>
       <c r="O37" s="11" t="inlineStr">
         <is>
-          <t>needs_mapping</t>
+          <t>source_available_unverified</t>
         </is>
       </c>
       <c r="P37" s="10" t="inlineStr">
@@ -4688,8 +4710,8 @@
       </c>
       <c r="R37" s="7" t="inlineStr">
         <is>
-          <t>скупой заправляет салат уксусом, философ добавляет в него соль, щедрый поливает его маслом. Что должен сделать четвертый повар-художник во время приготовления салата?
-Медиа из source_docs: Время.png.
+          <t>(Ее презентовала компания Кодак под лозунгом «Вы нажимаете на кнопку, мы делаем все остальное» - фото «Кодак-2»)
+Медиа из source_docs: Кодак-2.jpg.
 Резервная строка: использовать только после редакторского отбора.</t>
         </is>
       </c>
@@ -4705,7 +4727,7 @@
       </c>
       <c r="U37" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 2. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Время.png; не скопирован в app/static.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 4. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Кодак-2.jpg; не скопирован в app/static. Решение Виктора: Kodak-2 использовать как основной визуал; Kodak-1 не основной.</t>
         </is>
       </c>
       <c r="V37" s="9" t="inlineStr">
@@ -4722,11 +4744,11 @@
     </row>
     <row r="38" ht="95" customHeight="1">
       <c r="A38" s="9" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q041</t>
+          <t>v2_edited_q042</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
@@ -4741,7 +4763,7 @@
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>Перед вами рекламный плакат нового изобретения «Вы нажимаете на кнопку, мы делаем все остальное». В 2000 компания была лидером продаж. Что рекламировал данный плакат?</t>
+          <t>Открытие произошло совершенно случайно. Инженер придумал это, когда в его кармане растаяла конфета. Первая версия весила 300 килограмм и была двухметровой. Что изображено на схеме?</t>
         </is>
       </c>
       <c r="F38" s="7" t="n"/>
@@ -4750,10 +4772,10 @@
       <c r="I38" s="7" t="n"/>
       <c r="J38" s="9" t="inlineStr">
         <is>
-          <t>фотокамеру</t>
-        </is>
-      </c>
-      <c r="K38" s="9" t="inlineStr">
+          <t>микроволновая печь</t>
+        </is>
+      </c>
+      <c r="K38" s="21" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -4765,12 +4787,12 @@
       </c>
       <c r="M38" s="11" t="inlineStr">
         <is>
-          <t>v2_edited_kodak_2</t>
+          <t>v2_edited_microwave</t>
         </is>
       </c>
       <c r="N38" s="11" t="inlineStr">
         <is>
-          <t>v2_edited_kodak_2.jpg</t>
+          <t>v2_edited_microwave.jpg</t>
         </is>
       </c>
       <c r="O38" s="11" t="inlineStr">
@@ -4790,8 +4812,8 @@
       </c>
       <c r="R38" s="7" t="inlineStr">
         <is>
-          <t>(Ее презентовала компания Кодак под лозунгом «Вы нажимаете на кнопку, мы делаем все остальное» - фото «Кодак-2»)
-Медиа из source_docs: Кодак-2.jpg.
+          <t>Микроволновая печь. Пенсир Спенсер был специалистом по проектированию локационных приборов. Конфетка, лежащая в его кармане растаяла – так изобрели микроволновку.(Фото «Микроволновка»)
+Медиа из source_docs: Микроволновка.jpg.
 Резервная строка: использовать только после редакторского отбора.</t>
         </is>
       </c>
@@ -4807,7 +4829,7 @@
       </c>
       <c r="U38" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 4. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Кодак-2.jpg; не скопирован в app/static. Решение Виктора: Kodak-2 использовать как основной визуал; Kodak-1 не основной.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 5. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Микроволновка.jpg; не скопирован в app/static. Решение Виктора: микроволновка / растаявшая конфета — использовать как визуальный вопрос. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V38" s="9" t="inlineStr">
@@ -4824,11 +4846,11 @@
     </row>
     <row r="39" ht="95" customHeight="1">
       <c r="A39" s="9" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q042</t>
+          <t>v2_edited_q043</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -4843,7 +4865,7 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>Открытие произошло совершенно случайно. Инженер придумал это, когда в его кармане растаяла конфета. Первая версия весила 300 килограмм и была двухметровой. Что изображено на схеме?</t>
+          <t>Марка. На ней изображена Жозофина Кокрей. Которая изобрела полезную вещь. Но больше всего страдали служанки, потому что изобретение посягало на их работу. О чем идет речь?</t>
         </is>
       </c>
       <c r="F39" s="7" t="n"/>
@@ -4852,10 +4874,10 @@
       <c r="I39" s="7" t="n"/>
       <c r="J39" s="9" t="inlineStr">
         <is>
-          <t>микроволновая печь</t>
-        </is>
-      </c>
-      <c r="K39" s="21" t="inlineStr">
+          <t>посудомоечная машина</t>
+        </is>
+      </c>
+      <c r="K39" s="9" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -4867,12 +4889,12 @@
       </c>
       <c r="M39" s="11" t="inlineStr">
         <is>
-          <t>v2_edited_microwave</t>
+          <t>v2_edited_dishwasher</t>
         </is>
       </c>
       <c r="N39" s="11" t="inlineStr">
         <is>
-          <t>v2_edited_microwave.jpg</t>
+          <t>v2_edited_dishwasher.jfif</t>
         </is>
       </c>
       <c r="O39" s="11" t="inlineStr">
@@ -4892,8 +4914,8 @@
       </c>
       <c r="R39" s="7" t="inlineStr">
         <is>
-          <t>Микроволновая печь. Пенсир Спенсер был специалистом по проектированию локационных приборов. Конфетка, лежащая в его кармане растаяла – так изобрели микроволновку.(Фото «Микроволновка»)
-Медиа из source_docs: Микроволновка.jpg.
+          <t>В 1893 году она продемонстировала ее на выставке в Чикаго. Многие считали, что это против традиционных устоев. Прислуга же боялась, что эта машина оставит их без работы. (Фото «Посудомойка»)
+Медиа из source_docs: Посудомойка.jfif.
 Резервная строка: использовать только после редакторского отбора.</t>
         </is>
       </c>
@@ -4909,7 +4931,7 @@
       </c>
       <c r="U39" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 5. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Микроволновка.jpg; не скопирован в app/static. Решение Виктора: микроволновка / растаявшая конфета — использовать как визуальный вопрос. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 6. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Посудомойка.jfif; не скопирован в app/static. Решение Виктора: Жозефина Кокрейн / посудомоечная машина — использовать как визуальный вопрос.</t>
         </is>
       </c>
       <c r="V39" s="9" t="inlineStr">
@@ -4926,11 +4948,11 @@
     </row>
     <row r="40" ht="95" customHeight="1">
       <c r="A40" s="9" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q043</t>
+          <t>v2_edited_q044</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
@@ -4945,7 +4967,7 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>Марка. На ней изображена Жозофина Кокрей. Которая изобрела полезную вещь. Но больше всего страдали служанки, потому что изобретение посягало на их работу. О чем идет речь?</t>
+          <t>Представителям этой профессии обязательно нужны были кожаные перчатки. Часто они держали возле себя харьков или лис. О какой профессии идет речь?</t>
         </is>
       </c>
       <c r="F40" s="7" t="n"/>
@@ -4954,7 +4976,7 @@
       <c r="I40" s="7" t="n"/>
       <c r="J40" s="9" t="inlineStr">
         <is>
-          <t>посудомоечная машина</t>
+          <t>Крысолов.</t>
         </is>
       </c>
       <c r="K40" s="9" t="inlineStr">
@@ -4969,12 +4991,12 @@
       </c>
       <c r="M40" s="11" t="inlineStr">
         <is>
-          <t>v2_edited_dishwasher</t>
+          <t>v2_edited_ratcatcher_2</t>
         </is>
       </c>
       <c r="N40" s="11" t="inlineStr">
         <is>
-          <t>v2_edited_dishwasher.jfif</t>
+          <t>v2_edited_ratcatcher_2.jfif</t>
         </is>
       </c>
       <c r="O40" s="11" t="inlineStr">
@@ -4994,8 +5016,8 @@
       </c>
       <c r="R40" s="7" t="inlineStr">
         <is>
-          <t>В 1893 году она продемонстировала ее на выставке в Чикаго. Многие считали, что это против традиционных устоев. Прислуга же боялась, что эта машина оставит их без работы. (Фото «Посудомойка»)
-Медиа из source_docs: Посудомойка.jfif.
+          <t>Перчатки нужны были, чтобы защищать руки от укусов крыс. (Фото «Крысолов-2»)
+Медиа из source_docs: Крысолов-2.jfif.
 Резервная строка: использовать только после редакторского отбора.</t>
         </is>
       </c>
@@ -5011,7 +5033,7 @@
       </c>
       <c r="U40" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 6. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Посудомойка.jfif; не скопирован в app/static. Решение Виктора: Жозефина Кокрейн / посудомоечная машина — использовать как визуальный вопрос.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 7. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Крысолов-2.jfif; не скопирован в app/static.</t>
         </is>
       </c>
       <c r="V40" s="9" t="inlineStr">
@@ -5028,11 +5050,11 @@
     </row>
     <row r="41" ht="95" customHeight="1">
       <c r="A41" s="9" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q044</t>
+          <t>v2_edited_q045</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
@@ -5047,7 +5069,7 @@
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>Представителям этой профессии обязательно нужны были кожаные перчатки. Часто они держали возле себя харьков или лис. О какой профессии идет речь?</t>
+          <t>Женщина по имени Руд Бервиль. Ее товар нельзя купить ни за какие деньги. Свежий товар она получала благодаря королевской обсерватории в Гринвиче. Что продавала эта женщина?</t>
         </is>
       </c>
       <c r="F41" s="7" t="n"/>
@@ -5056,10 +5078,10 @@
       <c r="I41" s="7" t="n"/>
       <c r="J41" s="9" t="inlineStr">
         <is>
-          <t>Крысолов.</t>
-        </is>
-      </c>
-      <c r="K41" s="9" t="inlineStr">
+          <t>точное время</t>
+        </is>
+      </c>
+      <c r="K41" s="21" t="inlineStr">
         <is>
           <t>да</t>
         </is>
@@ -5071,12 +5093,12 @@
       </c>
       <c r="M41" s="11" t="inlineStr">
         <is>
-          <t>v2_edited_ratcatcher_2</t>
+          <t>v2_edited_time_seller</t>
         </is>
       </c>
       <c r="N41" s="11" t="inlineStr">
         <is>
-          <t>v2_edited_ratcatcher_2.jfif</t>
+          <t>v2_edited_time_seller.jpg</t>
         </is>
       </c>
       <c r="O41" s="11" t="inlineStr">
@@ -5096,8 +5118,8 @@
       </c>
       <c r="R41" s="7" t="inlineStr">
         <is>
-          <t>Перчатки нужны были, чтобы защищать руки от укусов крыс. (Фото «Крысолов-2»)
-Медиа из source_docs: Крысолов-2.jfif.
+          <t>Время. Точное время. За точным временем обращались часовщики, банкиры. Часы выставленные по гринвичевскому времени – были вопросом статуса и пользовалась успехом у клиентов.(Фото «Время»)
+Медиа из source_docs: Продавщица времени.jpg.
 Резервная строка: использовать только после редакторского отбора.</t>
         </is>
       </c>
@@ -5113,7 +5135,7 @@
       </c>
       <c r="U41" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 7. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Крысолов-2.jfif; не скопирован в app/static.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 8. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Продавщица времени.jpg; не скопирован в app/static. Решение Виктора: выбрать лучший вариант между Время.jpg и Продавщица времени.jpg после просмотра. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
         </is>
       </c>
       <c r="V41" s="9" t="inlineStr">
@@ -5130,11 +5152,11 @@
     </row>
     <row r="42" ht="95" customHeight="1">
       <c r="A42" s="9" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q045</t>
+          <t>v2_edited_q046</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
@@ -5144,12 +5166,12 @@
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>image_clue</t>
+          <t>reserve</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>Женщина по имени Руд Бервиль. Ее товар нельзя купить ни за какие деньги. Свежий товар она получала благодаря королевской обсерватории в Гринвиче. Что продавала эта женщина?</t>
+          <t>Как называется море, названное в честь двух родственников: Дмитрия Яковлевича (вице-адмирала) и Харитона Прокофьевича (капитана 1-го ранга).</t>
         </is>
       </c>
       <c r="F42" s="7" t="n"/>
@@ -5158,37 +5180,29 @@
       <c r="I42" s="7" t="n"/>
       <c r="J42" s="9" t="inlineStr">
         <is>
-          <t>точное время</t>
-        </is>
-      </c>
-      <c r="K42" s="21" t="inlineStr">
+          <t>Море Лаптевых</t>
+        </is>
+      </c>
+      <c r="K42" s="9" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="L42" s="10" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="M42" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_time_seller</t>
-        </is>
-      </c>
-      <c r="N42" s="11" t="inlineStr">
-        <is>
-          <t>v2_edited_time_seller.jpg</t>
-        </is>
-      </c>
-      <c r="O42" s="11" t="inlineStr">
-        <is>
-          <t>source_available_unverified</t>
-        </is>
-      </c>
-      <c r="P42" s="10" t="inlineStr">
-        <is>
-          <t>with_question</t>
+      <c r="L42" s="9" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M42" s="7" t="inlineStr"/>
+      <c r="N42" s="7" t="inlineStr"/>
+      <c r="O42" s="7" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="P42" s="9" t="inlineStr">
+        <is>
+          <t>none</t>
         </is>
       </c>
       <c r="Q42" s="7" t="inlineStr">
@@ -5198,9 +5212,7 @@
       </c>
       <c r="R42" s="7" t="inlineStr">
         <is>
-          <t>Время. Точное время. За точным временем обращались часовщики, банкиры. Часы выставленные по гринвичевскому времени – были вопросом статуса и пользовалась успехом у клиентов.(Фото «Время»)
-Медиа из source_docs: Продавщица времени.jpg.
-Резервная строка: использовать только после редакторского отбора.</t>
+          <t>Резервная строка: использовать только после редакторского отбора.</t>
         </is>
       </c>
       <c r="S42" s="9" t="inlineStr">
@@ -5208,14 +5220,14 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="T42" s="10" t="inlineStr">
-        <is>
-          <t>needs_media</t>
+      <c r="T42" s="12" t="inlineStr">
+        <is>
+          <t>needs_review</t>
         </is>
       </c>
       <c r="U42" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 8. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Продавщица времени.jpg; не скопирован в app/static. Решение Виктора: выбрать лучший вариант между Время.jpg и Продавщица времени.jpg после просмотра. | Правильный ответ заполнен из существующей заметки/вариантов; всё ещё нужен редакторский review.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 10. Аудит action=reserve. answer_type=open_answer.</t>
         </is>
       </c>
       <c r="V42" s="9" t="inlineStr">
@@ -5232,11 +5244,11 @@
     </row>
     <row r="43" ht="95" customHeight="1">
       <c r="A43" s="9" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q046</t>
+          <t>v2_edited_q047</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
@@ -5246,12 +5258,12 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>reserve</t>
+          <t>duel_question</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>Как называется море, названное в честь двух родственников: Дмитрия Яковлевича (вице-адмирала) и Харитона Прокофьевича (капитана 1-го ранга).</t>
+          <t>Слово «король» произошло в процессе адаптации имени Карла Великого. А от какого имени происходит слово «царь»?</t>
         </is>
       </c>
       <c r="F43" s="7" t="n"/>
@@ -5260,7 +5272,7 @@
       <c r="I43" s="7" t="n"/>
       <c r="J43" s="9" t="inlineStr">
         <is>
-          <t>Море Лаптевых</t>
+          <t>Цезарь</t>
         </is>
       </c>
       <c r="K43" s="9" t="inlineStr">
@@ -5307,7 +5319,7 @@
       </c>
       <c r="U43" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 10. Аудит action=reserve. answer_type=open_answer.</t>
+          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 11. Аудит action=reserve. answer_type=open_answer.</t>
         </is>
       </c>
       <c r="V43" s="9" t="inlineStr">
@@ -5324,11 +5336,11 @@
     </row>
     <row r="44" ht="95" customHeight="1">
       <c r="A44" s="9" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>v2_edited_q047</t>
+          <t>v2_edited_q048</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
@@ -5338,12 +5350,12 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>duel_question</t>
+          <t>image_clue</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>Слово «король» произошло в процессе адаптации имени Карла Великого. А от какого имени происходит слово «царь»?</t>
+          <t>Где в одном месте можно увидеть изображения Царя Давида, Александра Македонского, Юлия Цезаря и Карла Великого?</t>
         </is>
       </c>
       <c r="F44" s="7" t="n"/>
@@ -5352,7 +5364,7 @@
       <c r="I44" s="7" t="n"/>
       <c r="J44" s="9" t="inlineStr">
         <is>
-          <t>Цезарь</t>
+          <t>в классической колоде игральных карт.</t>
         </is>
       </c>
       <c r="K44" s="9" t="inlineStr">
@@ -5360,162 +5372,71 @@
           <t>да</t>
         </is>
       </c>
-      <c r="L44" s="9" t="inlineStr">
+      <c r="L44" s="21" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="M44" s="20" t="inlineStr">
+        <is>
+          <t>v2_edited_card_kings</t>
+        </is>
+      </c>
+      <c r="N44" s="20" t="inlineStr">
+        <is>
+          <t>v2_edited_card_kings.jpg</t>
+        </is>
+      </c>
+      <c r="O44" s="20" t="inlineStr">
+        <is>
+          <t>needs_clean_source</t>
+        </is>
+      </c>
+      <c r="P44" s="21" t="inlineStr">
+        <is>
+          <t>with_question</t>
+        </is>
+      </c>
+      <c r="Q44" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="M44" s="7" t="inlineStr"/>
-      <c r="N44" s="7" t="inlineStr"/>
-      <c r="O44" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="P44" s="9" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="Q44" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
       <c r="R44" s="7" t="inlineStr">
-        <is>
-          <t>Резервная строка: использовать только после редакторского отбора.</t>
-        </is>
-      </c>
-      <c r="S44" s="9" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="T44" s="12" t="inlineStr">
-        <is>
-          <t>needs_review</t>
-        </is>
-      </c>
-      <c r="U44" s="7" t="inlineStr">
-        <is>
-          <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 11. Аудит action=reserve. answer_type=open_answer.</t>
-        </is>
-      </c>
-      <c r="V44" s="9" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="W44" s="9" t="inlineStr">
-        <is>
-          <t>НЕТ (no, not_ready)</t>
-        </is>
-      </c>
-      <c r="X44" s="7" t="inlineStr"/>
-    </row>
-    <row r="45" ht="95" customHeight="1">
-      <c r="A45" s="9" t="n">
-        <v>48</v>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>v2_edited_q048</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>v2_reserve</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>image_clue</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>Где в одном месте можно увидеть изображения Царя Давида, Александра Македонского, Юлия Цезаря и Карла Великого?</t>
-        </is>
-      </c>
-      <c r="F45" s="7" t="n"/>
-      <c r="G45" s="7" t="n"/>
-      <c r="H45" s="7" t="n"/>
-      <c r="I45" s="7" t="n"/>
-      <c r="J45" s="9" t="inlineStr">
-        <is>
-          <t>в классической колоде игральных карт.</t>
-        </is>
-      </c>
-      <c r="K45" s="9" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="L45" s="21" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="M45" s="20" t="inlineStr">
-        <is>
-          <t>v2_edited_card_kings</t>
-        </is>
-      </c>
-      <c r="N45" s="20" t="inlineStr">
-        <is>
-          <t>v2_edited_card_kings.jpg</t>
-        </is>
-      </c>
-      <c r="O45" s="20" t="inlineStr">
-        <is>
-          <t>needs_clean_source</t>
-        </is>
-      </c>
-      <c r="P45" s="21" t="inlineStr">
-        <is>
-          <t>with_question</t>
-        </is>
-      </c>
-      <c r="Q45" s="7" t="inlineStr">
-        <is>
-          <t>нет</t>
-        </is>
-      </c>
-      <c r="R45" s="7" t="inlineStr">
         <is>
           <t>(Эти исторические личности стали прототипами изображений королей на лицевой стороне карточной колоды. – Фото «Короли карты»)
 Медиа из source_docs: Короли-карты.jpg.
 Резервная строка: использовать только после редакторского отбора.</t>
         </is>
       </c>
-      <c r="S45" s="9" t="inlineStr">
+      <c r="S44" s="9" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="T45" s="21" t="inlineStr">
+      <c r="T44" s="21" t="inlineStr">
         <is>
           <t>needs_clean_source</t>
         </is>
       </c>
-      <c r="U45" s="7" t="inlineStr">
+      <c r="U44" s="7" t="inlineStr">
         <is>
           <t>Источник: edited DOCX, раздел "ВОПРОСЫ БЕЗ ВАРИАНТОВ:", № 12. Аудит action=needs_media. answer_type=open_answer. risk_flags=needs_media. Исходный asset есть в docs/question_bank_v2/source_docs/Короли-карты.jpg; не скопирован в app/static. Решение Виктора: Короли-карты.jpg требует clean source; текущий файл похож на изображение с источником/водяным знаком.</t>
         </is>
       </c>
-      <c r="V45" s="9" t="inlineStr">
+      <c r="V44" s="9" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="W45" s="9" t="inlineStr">
+      <c r="W44" s="9" t="inlineStr">
         <is>
           <t>НЕТ (no, not_ready)</t>
         </is>
       </c>
-      <c r="X45" s="7" t="inlineStr"/>
-    </row>
+      <c r="X44" s="7" t="inlineStr"/>
+    </row>
+    <row r="45" ht="95" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:X45"/>
   <dataValidations count="1">
@@ -5534,7 +5455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5694,6 +5615,36 @@
       <c r="F5" s="7" t="inlineStr">
         <is>
           <t>НЕТ (no, not_ready)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>v2_edited_q001</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>v2_warmup_oath</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>plain_text</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>В белорусской столице Минске установлен памятник картошке.</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
         </is>
       </c>
     </row>
@@ -6254,7 +6205,7 @@
       </c>
       <c r="K2" s="7" t="inlineStr"/>
       <c r="L2" s="7" t="inlineStr"/>
-      <c r="M2" s="7" t="inlineStr"/>
+      <c r="M2" s="7" t="n"/>
       <c r="N2" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -6293,7 +6244,7 @@
       </c>
       <c r="V2" s="7" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>cut</t>
         </is>
       </c>
       <c r="W2" s="7" t="inlineStr">
@@ -6314,7 +6265,7 @@
       </c>
       <c r="AA2" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 6. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 6. Аудит action=keep. answer_type=true_false. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. Правильный ответ ещё нужно подтвердить/заполнить. | Victor decision: cut. Формулировка “в Минске установлен памятник картошке” не подтверждена надёжно; подтверждаются памятники картошке в Беларуси/Минской области, но не в столице Минске.</t>
         </is>
       </c>
     </row>
@@ -6942,7 +6893,11 @@
       </c>
       <c r="K8" s="7" t="inlineStr"/>
       <c r="L8" s="7" t="inlineStr"/>
-      <c r="M8" s="7" t="inlineStr"/>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -6994,7 +6949,7 @@
       </c>
       <c r="AA8" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 12. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 12. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить. | Victor decision: answer=правда. Слово “сарай” восходит к персидскому/иранскому слову со значением дворец, дом, помещение; формулировку лучше смягчить.</t>
         </is>
       </c>
     </row>
@@ -7047,7 +7002,11 @@
       </c>
       <c r="K9" s="7" t="inlineStr"/>
       <c r="L9" s="7" t="inlineStr"/>
-      <c r="M9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>правда</t>
+        </is>
+      </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -7099,7 +7058,7 @@
       </c>
       <c r="AA9" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 13. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ПРАВДА ИЛИ ПИЗДЁЖ?", № 13. Аудит action=keep. answer_type=true_false. Правильный ответ ещё нужно подтвердить/заполнить. | Victor decision: answer=правда. Это не постоянная служба, а рождественская горячая линия/helpline Hasbro UK/Ireland для споров по Monopoly.</t>
         </is>
       </c>
     </row>
@@ -9453,7 +9412,7 @@
           <t>просто отодвинул затвор</t>
         </is>
       </c>
-      <c r="M30" s="7" t="inlineStr"/>
+      <c r="M30" s="7" t="n"/>
       <c r="N30" s="7" t="inlineStr">
         <is>
           <t>image</t>
@@ -9514,7 +9473,7 @@
       </c>
       <c r="AA30" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 14. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. Решение Виктора: Кеша из Блудного попугая пока не финализировать; нужен точный кадр/видео. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 14. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. Решение Виктора: Кеша из Блудного попугая пока не финализировать; нужен точный кадр/видео. Правильный ответ ещё нужно подтвердить/заполнить. | Victor decision: keep reserve; preliminary option D — просто отодвинул затвор. Финальный ответ ставить только после проверки кадра/видео.</t>
         </is>
       </c>
     </row>
@@ -10451,7 +10410,11 @@
           <t>расческа</t>
         </is>
       </c>
-      <c r="M38" s="7" t="inlineStr"/>
+      <c r="M38" s="7" t="inlineStr">
+        <is>
+          <t>зубная щётка</t>
+        </is>
+      </c>
       <c r="N38" s="7" t="inlineStr">
         <is>
           <t>none</t>
@@ -10507,7 +10470,7 @@
       </c>
       <c r="AA38" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 22. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: предмет гигиены через армию — reserve/source_check. Правильный ответ ещё нужно подтвердить/заполнить.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 22. Аудит action=rewrite. answer_type=multiple_choice. Решение Виктора: предмет гигиены через армию — reserve/source_check. Правильный ответ ещё нужно подтвердить/заполнить. | Victor decision: answer=зубная щётка. Reserve/source_check; формулировку надо смягчить.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close question bank v2 row 29 as reserve
</commit_message>
<xml_diff>
--- a/docs/question_bank_v2/question_bank_v2_authoring_draft.xlsx
+++ b/docs/question_bank_v2/question_bank_v2_authoring_draft.xlsx
@@ -3362,7 +3362,7 @@
       <c r="J25" s="9" t="n"/>
       <c r="K25" s="21" t="inlineStr">
         <is>
-          <t>НЕТ — проверить видео/кадр</t>
+          <t>резерв — не блокирует игру</t>
         </is>
       </c>
       <c r="L25" s="10" t="inlineStr">
@@ -3394,7 +3394,7 @@
       <c r="R25" s="7" t="inlineStr">
         <is>
           <t>(Тут нужна картинка на ответ или видео)
-Медиа из source_docs: проверить файл в source_docs. | Предварительный вариант по решению Виктора: D — просто отодвинул затвор. Финальный ответ ставить только после проверки кадра/видео.</t>
+Медиа из source_docs: проверить файл в source_docs. | Предварительный вариант по решению Виктора: D — просто отодвинул затвор. Финальный ответ ставить только после проверки кадра/видео. | Reserve-only по решению Виктора: не блокирует подготовку коммерческой игры; можно вернуться после проверки кадра/видео. Предварительная версия: D — просто отодвинул затвор, не финальный ответ.</t>
         </is>
       </c>
       <c r="S25" s="9" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 14. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. Решение Виктора: Кеша из Блудного попугая пока не финализировать; нужен точный кадр/видео. | Reserve. Проверить точный кадр/видео; до проверки финальный ответ не заполнять.</t>
+          <t>не блокирует подготовку; можно вернуться после проверки кадра/видео</t>
         </is>
       </c>
       <c r="V25" s="9" t="inlineStr">
@@ -3422,7 +3422,11 @@
           <t>НЕТ (no, not_ready)</t>
         </is>
       </c>
-      <c r="X25" s="7" t="inlineStr"/>
+      <c r="X25" s="7" t="inlineStr">
+        <is>
+          <t>Не включать в финальный активный/import candidate set до проверки видео.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="95" customHeight="1">
       <c r="A26" s="9" t="n">
@@ -9473,7 +9477,7 @@
       </c>
       <c r="AA30" s="7" t="inlineStr">
         <is>
-          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 14. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. Решение Виктора: Кеша из Блудного попугая пока не финализировать; нужен точный кадр/видео. Правильный ответ ещё нужно подтвердить/заполнить. | Victor decision: keep reserve; preliminary option D — просто отодвинул затвор. Финальный ответ ставить только после проверки кадра/видео.</t>
+          <t>Источник: edited DOCX, раздел "ВАРИАНТЫ ОТВЕТОВ:", № 14. Аудит action=needs_media. answer_type=multiple_choice. risk_flags=needs_media. Медиа требуется подобрать/проверить; в app/static не копировалось. Решение Виктора: Кеша из Блудного попугая пока не финализировать; нужен точный кадр/видео. Правильный ответ ещё нужно подтвердить/заполнить. | Victor decision: keep reserve; preliminary option D — просто отодвинул затвор. Финальный ответ ставить только после проверки кадра/видео. | Victor decision: close as reserve-only for current commercial game preparation. Keep needs_video_check; preliminary D — просто отодвинул затвор remains non-final note; correct_answer_draft intentionally empty.</t>
         </is>
       </c>
     </row>

</xml_diff>